<commit_message>
Add refund management workflow and export support
</commit_message>
<xml_diff>
--- a/provident-system/server/uploads/templates/sl.xlsx
+++ b/provident-system/server/uploads/templates/sl.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000"/>
+    <workbookView windowWidth="22188" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="JUNE 2026 " sheetId="1" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="192">
   <si>
     <t>SUBSIDIARY LEDGER</t>
   </si>
@@ -201,6 +201,441 @@
   </si>
   <si>
     <t>2026-06-4256</t>
+  </si>
+  <si>
+    <t>RIVERA, ERLYN P.</t>
+  </si>
+  <si>
+    <t>PASIG NHS/ CANDABA</t>
+  </si>
+  <si>
+    <t>0085104721</t>
+  </si>
+  <si>
+    <t>2026-06-4257</t>
+  </si>
+  <si>
+    <t>PABUSTAN, REGIE S.</t>
+  </si>
+  <si>
+    <t>SDO PAMPANGA</t>
+  </si>
+  <si>
+    <t>0085202898</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>2026-06-4258</t>
+  </si>
+  <si>
+    <t>5422402</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>ADA-III</t>
+  </si>
+  <si>
+    <t>13071</t>
+  </si>
+  <si>
+    <t>4336279</t>
+  </si>
+  <si>
+    <t>New</t>
+  </si>
+  <si>
+    <t>ADDITIONAL</t>
+  </si>
+  <si>
+    <t>2026-06-4259</t>
+  </si>
+  <si>
+    <t>BACANI, HENRY B.</t>
+  </si>
+  <si>
+    <t>095</t>
+  </si>
+  <si>
+    <t>5410694</t>
+  </si>
+  <si>
+    <t>ADA-I</t>
+  </si>
+  <si>
+    <t>TEOPACO, ANALISA S.</t>
+  </si>
+  <si>
+    <t>5422401</t>
+  </si>
+  <si>
+    <t>Additional</t>
+  </si>
+  <si>
+    <t>0085205021</t>
+  </si>
+  <si>
+    <t>2026-06-4260</t>
+  </si>
+  <si>
+    <t>MUSNI, ENGELYN S.</t>
+  </si>
+  <si>
+    <t>018</t>
+  </si>
+  <si>
+    <t>5407386</t>
+  </si>
+  <si>
+    <t>AO-II</t>
+  </si>
+  <si>
+    <t>13072</t>
+  </si>
+  <si>
+    <t>STA. CATALINA ES/ SAN LUIS</t>
+  </si>
+  <si>
+    <t>ROS, GLENDA B.</t>
+  </si>
+  <si>
+    <t>4160293</t>
+  </si>
+  <si>
+    <t>0085203185</t>
+  </si>
+  <si>
+    <t>RENEWAL</t>
+  </si>
+  <si>
+    <t>2026-06-4261</t>
+  </si>
+  <si>
+    <t>36</t>
+  </si>
+  <si>
+    <t>13073</t>
+  </si>
+  <si>
+    <t>NICDAO, NOEMI G.</t>
+  </si>
+  <si>
+    <t>4160620</t>
+  </si>
+  <si>
+    <t>Renewal</t>
+  </si>
+  <si>
+    <t>2908171</t>
+  </si>
+  <si>
+    <t>JUNE</t>
+  </si>
+  <si>
+    <t>0085207393</t>
+  </si>
+  <si>
+    <t>2026-06-4262</t>
+  </si>
+  <si>
+    <t>DE JESUS, VICTORIA CORAZON P.</t>
+  </si>
+  <si>
+    <t>536</t>
+  </si>
+  <si>
+    <t>4162627</t>
+  </si>
+  <si>
+    <t>48</t>
+  </si>
+  <si>
+    <t>13074</t>
+  </si>
+  <si>
+    <t>SALAPUNGAN NHS/ CANDABA</t>
+  </si>
+  <si>
+    <t>ANDAL, IRENE C.</t>
+  </si>
+  <si>
+    <t>4594536</t>
+  </si>
+  <si>
+    <t>2908080</t>
+  </si>
+  <si>
+    <t>0105089473</t>
+  </si>
+  <si>
+    <t>2026-06-4263</t>
+  </si>
+  <si>
+    <t>REYES, MA. LUISA M.</t>
+  </si>
+  <si>
+    <t>T-III</t>
+  </si>
+  <si>
+    <t>SAN ISIDRO ES/ SAN LUIS</t>
+  </si>
+  <si>
+    <t>0085181793</t>
+  </si>
+  <si>
+    <t>2026-06-4264</t>
+  </si>
+  <si>
+    <t>BALLESTEROS, IRAH S.</t>
+  </si>
+  <si>
+    <t>039</t>
+  </si>
+  <si>
+    <t>STA. LUTGARDA ES/ MACABEBE WEST</t>
+  </si>
+  <si>
+    <t>CABRERA, GLAIZA G.</t>
+  </si>
+  <si>
+    <t>3425048979</t>
+  </si>
+  <si>
+    <t>2026-06-4265</t>
+  </si>
+  <si>
+    <t>ISIP, ALMA M.</t>
+  </si>
+  <si>
+    <t>STO. NINO ES/ MACABEBE WEST</t>
+  </si>
+  <si>
+    <t>3425048464</t>
+  </si>
+  <si>
+    <t>2026-06-4266</t>
+  </si>
+  <si>
+    <t>LAURETA, ALMER A.</t>
+  </si>
+  <si>
+    <t>013</t>
+  </si>
+  <si>
+    <t>MASAMAT ES/ MEXICO SOUTH</t>
+  </si>
+  <si>
+    <t>LAURETA, EVELYN L.</t>
+  </si>
+  <si>
+    <t>0085142275</t>
+  </si>
+  <si>
+    <t>2026-06-4267</t>
+  </si>
+  <si>
+    <t>CANILAO, CATHERINE O.</t>
+  </si>
+  <si>
+    <t>MT-II</t>
+  </si>
+  <si>
+    <t>DALCUIS HS</t>
+  </si>
+  <si>
+    <t>SORIANO, RODERICK G.</t>
+  </si>
+  <si>
+    <t>0085072420</t>
+  </si>
+  <si>
+    <t>2026-06-4268</t>
+  </si>
+  <si>
+    <t>MUTUC, ANGELINA M.</t>
+  </si>
+  <si>
+    <t>HENSON ES/ PORAC EAST</t>
+  </si>
+  <si>
+    <t>0085095749</t>
+  </si>
+  <si>
+    <t>2026-06-4269</t>
+  </si>
+  <si>
+    <t>TAYAG, GLADYS R.</t>
+  </si>
+  <si>
+    <t>028</t>
+  </si>
+  <si>
+    <t>5410683</t>
+  </si>
+  <si>
+    <t>13075</t>
+  </si>
+  <si>
+    <t>DON MACARIO BACANI ES/ LUBAO NORTH</t>
+  </si>
+  <si>
+    <t>CRUZ, MIRELLA A.</t>
+  </si>
+  <si>
+    <t>4160142</t>
+  </si>
+  <si>
+    <t>3865018850</t>
+  </si>
+  <si>
+    <t>2026-06-4270</t>
+  </si>
+  <si>
+    <t>ARCE, FILAMER G.</t>
+  </si>
+  <si>
+    <t>505</t>
+  </si>
+  <si>
+    <t>5422404</t>
+  </si>
+  <si>
+    <t>13076</t>
+  </si>
+  <si>
+    <t>STA. CRUZ ES/ LUBAO WEST</t>
+  </si>
+  <si>
+    <t>BACANI, JOCELYN M.</t>
+  </si>
+  <si>
+    <t>4151281</t>
+  </si>
+  <si>
+    <t>3865021355</t>
+  </si>
+  <si>
+    <t>2026-06-4271</t>
+  </si>
+  <si>
+    <t>MANALASTAS, JENNETH P.</t>
+  </si>
+  <si>
+    <t>531</t>
+  </si>
+  <si>
+    <t>4264311</t>
+  </si>
+  <si>
+    <t>ADAS-II</t>
+  </si>
+  <si>
+    <t>13077</t>
+  </si>
+  <si>
+    <t>DY, JOYCE P.</t>
+  </si>
+  <si>
+    <t>4263339</t>
+  </si>
+  <si>
+    <t>2908121</t>
+  </si>
+  <si>
+    <t>3775017855</t>
+  </si>
+  <si>
+    <t>2026-06-4272</t>
+  </si>
+  <si>
+    <t>DAVID, JAYPEE D.</t>
+  </si>
+  <si>
+    <t>027</t>
+  </si>
+  <si>
+    <t>4160342</t>
+  </si>
+  <si>
+    <t>13078</t>
+  </si>
+  <si>
+    <t>MITLA ES/ PORAC WEST</t>
+  </si>
+  <si>
+    <t>TAMAYO, KRISTINE M.</t>
+  </si>
+  <si>
+    <t>4673906</t>
+  </si>
+  <si>
+    <t>2908079</t>
+  </si>
+  <si>
+    <t>1525056267</t>
+  </si>
+  <si>
+    <t>2026-06-4273</t>
+  </si>
+  <si>
+    <t>REYES, DWIGHT MICHAEL ANGELO A.</t>
+  </si>
+  <si>
+    <t>5419321</t>
+  </si>
+  <si>
+    <t>13079</t>
+  </si>
+  <si>
+    <t>MALLARI, JONATHAN CHRISTIAN P.</t>
+  </si>
+  <si>
+    <t>4160850</t>
+  </si>
+  <si>
+    <t>0085205153</t>
+  </si>
+  <si>
+    <t>2026-06-4274</t>
+  </si>
+  <si>
+    <t>2026-06-4275</t>
+  </si>
+  <si>
+    <t>SALARY</t>
+  </si>
+  <si>
+    <t>2026-06-4276</t>
+  </si>
+  <si>
+    <t>LENON, ALF M.</t>
+  </si>
+  <si>
+    <t>SALARY (MAY)</t>
+  </si>
+  <si>
+    <t>2026-06-4277</t>
+  </si>
+  <si>
+    <t>REYES, ROILANA M.</t>
+  </si>
+  <si>
+    <t>4261721</t>
+  </si>
+  <si>
+    <t>13080</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>0085135996</t>
   </si>
 </sst>
 </file>
@@ -216,7 +651,7 @@
     <numFmt numFmtId="177" formatCode="dd\-mmm\-yy"/>
     <numFmt numFmtId="178" formatCode="mmm\-yy"/>
   </numFmts>
-  <fonts count="40">
+  <fonts count="43">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -355,6 +790,29 @@
       <b/>
       <sz val="12"/>
       <color rgb="FF0C0C0C"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF002060"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -504,18 +962,18 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="9"/>
       <name val="Tahoma"/>
       <charset val="134"/>
     </font>
     <font>
-      <b/>
       <sz val="9"/>
       <name val="Tahoma"/>
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -524,7 +982,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -715,7 +1185,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -736,6 +1206,60 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="hair">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="hair">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="hair">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="hair">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="hair">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="hair">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="hair">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -839,31 +1363,19 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -872,318 +1384,414 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="6" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="7" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="7" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="8" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="104">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="176" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="1" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="176" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="176" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="176" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="176" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="177" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="176" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="176" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="10" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="176" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="176" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="176" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="176" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="176" fontId="8" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="177" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="176" fontId="10" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="176" fontId="16" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="17" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="4" fontId="17" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="43" fontId="18" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="43" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="43" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="43" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="43" fontId="16" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="43" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="43" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="43" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="176" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="10" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="176" fontId="11" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="176" fontId="12" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="176" fontId="10" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="176" fontId="16" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="3" fontId="17" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="4" fontId="17" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="43" fontId="18" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="43" fontId="12" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="43" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="43" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1237,221 +1845,29 @@
     <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
     <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="2">
     <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="double">
-          <color theme="4"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="0"/>
+        <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4"/>
-          <bgColor theme="4"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <border>
-        <left style="thin">
-          <color theme="4"/>
-        </left>
-        <right style="thin">
-          <color theme="4"/>
-        </right>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-        <horizontal style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
   </dxfs>
-  <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
-    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
-      <tableStyleElement type="wholeTable" dxfId="6"/>
-      <tableStyleElement type="headerRow" dxfId="5"/>
-      <tableStyleElement type="totalRow" dxfId="4"/>
-      <tableStyleElement type="firstColumn" dxfId="3"/>
-      <tableStyleElement type="lastColumn" dxfId="2"/>
-      <tableStyleElement type="firstRowStripe" dxfId="1"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
-    </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
-      <tableStyleElement type="headerRow" dxfId="16"/>
-      <tableStyleElement type="totalRow" dxfId="15"/>
-      <tableStyleElement type="firstRowStripe" dxfId="14"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
-      <tableStyleElement type="pageFieldValues" dxfId="7"/>
-    </tableStyle>
-  </tableStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1712,71 +2128,70 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:AD19"/>
+  <dimension ref="A1:AD40"/>
   <sheetFormatPr defaultColWidth="14.4444444444444" defaultRowHeight="15.6" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="8.22222222222222" style="1" customWidth="1"/>
-    <col min="2" max="2" width="33.6666666666667" style="2" customWidth="1"/>
-    <col min="3" max="3" width="10.1111111111111" style="1" customWidth="1"/>
-    <col min="4" max="4" width="15.8888888888889" style="1" customWidth="1"/>
-    <col min="5" max="5" width="40" style="1" customWidth="1"/>
-    <col min="6" max="6" width="28.3333333333333" style="3" customWidth="1"/>
-    <col min="7" max="7" width="25.3333333333333" style="1" customWidth="1"/>
-    <col min="8" max="8" width="16" style="4" customWidth="1"/>
-    <col min="9" max="9" width="14.5555555555556" style="4" customWidth="1"/>
-    <col min="10" max="10" width="18.8888888888889" style="1" customWidth="1"/>
-    <col min="11" max="11" width="19.6666666666667" style="1" customWidth="1"/>
-    <col min="12" max="12" width="15.3333333333333" style="1" customWidth="1"/>
-    <col min="13" max="13" width="14.8888888888889" style="1" hidden="1" customWidth="1"/>
-    <col min="14" max="14" width="15.3333333333333" style="1" hidden="1" customWidth="1"/>
-    <col min="15" max="15" width="13.4444444444444" style="1" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="15.3333333333333" style="1" hidden="1" customWidth="1"/>
-    <col min="17" max="17" width="10.2222222222222" style="5" customWidth="1"/>
-    <col min="18" max="18" width="14.7777777777778" style="1" customWidth="1"/>
-    <col min="19" max="19" width="14.6666666666667" style="1" customWidth="1"/>
-    <col min="20" max="20" width="13" style="6" customWidth="1"/>
-    <col min="21" max="21" width="14.8888888888889" style="2" customWidth="1"/>
-    <col min="22" max="22" width="11.2222222222222" style="7" customWidth="1"/>
-    <col min="23" max="23" width="56.1111111111111" style="1" customWidth="1"/>
-    <col min="24" max="24" width="38.2222222222222" style="1" customWidth="1"/>
-    <col min="25" max="25" width="16" style="5" customWidth="1"/>
-    <col min="26" max="26" width="41.1111111111111" style="1" customWidth="1"/>
-    <col min="27" max="27" width="27.7777777777778" style="8" customWidth="1"/>
-    <col min="28" max="28" width="18.2222222222222" style="1" customWidth="1"/>
-    <col min="29" max="29" width="16" style="9" customWidth="1"/>
-    <col min="30" max="30" width="23.5555555555556" style="1" customWidth="1"/>
-    <col min="31" max="31" width="15.3333333333333" style="1" customWidth="1"/>
-    <col min="32" max="32" width="24.8888888888889" style="1" customWidth="1"/>
-    <col min="33" max="16384" width="14.4444444444444" style="1" customWidth="1"/>
+    <col min="1" max="1" width="8.22222222222222" style="3" customWidth="1"/>
+    <col min="2" max="2" width="33.6666666666667" style="4" customWidth="1"/>
+    <col min="3" max="3" width="10.1111111111111" style="3" customWidth="1"/>
+    <col min="4" max="4" width="15.8888888888889" style="3" customWidth="1"/>
+    <col min="5" max="5" width="40" style="3" customWidth="1"/>
+    <col min="6" max="6" width="28.3333333333333" style="5" customWidth="1"/>
+    <col min="7" max="7" width="25.3333333333333" style="3" customWidth="1"/>
+    <col min="8" max="8" width="16" style="6" customWidth="1"/>
+    <col min="9" max="9" width="14.5555555555556" style="6" customWidth="1"/>
+    <col min="10" max="10" width="18.8888888888889" style="3" customWidth="1"/>
+    <col min="11" max="11" width="19.6666666666667" style="3" customWidth="1"/>
+    <col min="12" max="12" width="15.3333333333333" style="3" customWidth="1"/>
+    <col min="13" max="13" width="14.8888888888889" style="3" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="15.3333333333333" style="3" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="13.4444444444444" style="3" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="15.3333333333333" style="3" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="10.2222222222222" style="7" customWidth="1"/>
+    <col min="18" max="18" width="14.7777777777778" style="3" customWidth="1"/>
+    <col min="19" max="19" width="14.6666666666667" style="3" customWidth="1"/>
+    <col min="20" max="20" width="13" style="8" customWidth="1"/>
+    <col min="21" max="21" width="14.8888888888889" style="4" customWidth="1"/>
+    <col min="22" max="22" width="11.2222222222222" style="9" customWidth="1"/>
+    <col min="23" max="23" width="56.1111111111111" style="3" customWidth="1"/>
+    <col min="24" max="24" width="38.2222222222222" style="3" customWidth="1"/>
+    <col min="25" max="25" width="16" style="7" customWidth="1"/>
+    <col min="26" max="26" width="41.1111111111111" style="3" customWidth="1"/>
+    <col min="27" max="27" width="27.7777777777778" style="9" customWidth="1"/>
+    <col min="28" max="28" width="18.2222222222222" style="3" customWidth="1"/>
+    <col min="29" max="29" width="16" style="10" customWidth="1"/>
+    <col min="30" max="30" width="23.5555555555556" style="3" customWidth="1"/>
+    <col min="31" max="31" width="15.3333333333333" style="3" customWidth="1"/>
+    <col min="32" max="32" width="24.8888888888889" style="3" customWidth="1"/>
+    <col min="33" max="16384" width="14.4444444444444" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24.75" customHeight="1" spans="1:30">
-      <c r="A1" s="10"/>
-      <c r="B1" s="11" t="s">
+      <c r="A1" s="11"/>
+      <c r="B1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="12"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="G1" s="13"/>
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="10"/>
-      <c r="M1" s="10" t="s">
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="N1" s="10"/>
-      <c r="O1" s="10"/>
-      <c r="P1" s="10"/>
+      <c r="N1" s="11"/>
+      <c r="O1" s="11"/>
+      <c r="P1" s="11"/>
     </row>
     <row r="2" ht="6" customHeight="1" spans="1:30">
-      <c r="A2" s="10"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
       <c r="E2" s="15"/>
       <c r="F2" s="16"/>
       <c r="G2" s="17"/>
@@ -1786,35 +2201,34 @@
       <c r="K2" s="20"/>
       <c r="L2" s="21"/>
       <c r="M2" s="22"/>
-      <c r="N2" s="10"/>
+      <c r="N2" s="11"/>
       <c r="O2" s="19"/>
-      <c r="P2" s="10"/>
+      <c r="P2" s="11"/>
     </row>
     <row r="3" ht="36" customHeight="1" spans="1:30">
-      <c r="A3" s="10"/>
-      <c r="B3" s="11" t="s">
+      <c r="A3" s="11"/>
+      <c r="B3" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="12"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="G3" s="13"/>
       <c r="H3" s="14"/>
       <c r="I3" s="14"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
-      <c r="L3" s="12"/>
-      <c r="M3" s="12"/>
-      <c r="N3" s="10"/>
-      <c r="O3" s="10"/>
-      <c r="P3" s="10"/>
+      <c r="J3" s="13"/>
+      <c r="K3" s="13"/>
+      <c r="L3" s="13"/>
+      <c r="M3" s="13"/>
+      <c r="N3" s="11"/>
+      <c r="O3" s="11"/>
+      <c r="P3" s="11"/>
     </row>
     <row r="4" ht="22.95" customHeight="1" spans="1:30">
-      <c r="A4" s="10"/>
-      <c r="B4" s="11"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
+      <c r="A4" s="11"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
       <c r="E4" s="15"/>
       <c r="F4" s="16"/>
       <c r="G4" s="23">
@@ -1828,7 +2242,7 @@
       <c r="M4" s="22"/>
       <c r="N4" s="22"/>
       <c r="O4" s="19"/>
-      <c r="P4" s="10"/>
+      <c r="P4" s="11"/>
       <c r="Q4" s="24" t="s">
         <v>3</v>
       </c>
@@ -1920,13 +2334,13 @@
       <c r="AA5" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="AB5" s="37" t="s">
+      <c r="AB5" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="AC5" s="38" t="s">
+      <c r="AC5" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="AD5" s="1" t="s">
+      <c r="AD5" s="3" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1941,7 +2355,7 @@
       <c r="H6" s="18"/>
       <c r="I6" s="33"/>
       <c r="J6" s="33"/>
-      <c r="K6" s="39">
+      <c r="K6" s="37">
         <v>6245885.55000001</v>
       </c>
       <c r="L6" s="29"/>
@@ -1949,22 +2363,21 @@
       <c r="N6" s="29"/>
       <c r="O6" s="33"/>
       <c r="P6" s="29"/>
-      <c r="Q6" s="40"/>
-      <c r="R6" s="41"/>
-      <c r="S6" s="42"/>
-      <c r="T6" s="43"/>
-      <c r="U6" s="41"/>
-      <c r="V6" s="44"/>
-      <c r="W6" s="41"/>
-      <c r="X6" s="41"/>
-      <c r="Y6" s="40"/>
-      <c r="Z6" s="41"/>
+      <c r="Q6" s="24"/>
+      <c r="R6" s="25"/>
+      <c r="S6" s="36"/>
+      <c r="T6" s="26"/>
+      <c r="U6" s="25"/>
+      <c r="V6" s="27"/>
+      <c r="W6" s="25"/>
+      <c r="X6" s="25"/>
+      <c r="Y6" s="24"/>
+      <c r="Z6" s="25"/>
       <c r="AA6" s="27"/>
-      <c r="AB6" s="37"/>
-      <c r="AC6" s="38"/>
+      <c r="AC6" s="28"/>
     </row>
     <row r="7" ht="13.5" customHeight="1" spans="1:30">
-      <c r="A7" s="45"/>
+      <c r="A7" s="38"/>
       <c r="B7" s="30"/>
       <c r="C7" s="29"/>
       <c r="D7" s="29"/>
@@ -1975,138 +2388,134 @@
       </c>
       <c r="H7" s="18"/>
       <c r="I7" s="18"/>
-      <c r="J7" s="46"/>
-      <c r="K7" s="39">
+      <c r="J7" s="39"/>
+      <c r="K7" s="37">
         <v>6245885.55000001</v>
       </c>
-      <c r="L7" s="46"/>
+      <c r="L7" s="39"/>
       <c r="M7" s="35"/>
       <c r="N7" s="29"/>
-      <c r="O7" s="46"/>
+      <c r="O7" s="39"/>
       <c r="P7" s="29"/>
       <c r="Q7" s="26"/>
       <c r="R7" s="20"/>
       <c r="S7" s="20"/>
       <c r="T7" s="26"/>
       <c r="U7" s="17"/>
-      <c r="V7" s="47"/>
+      <c r="V7" s="40"/>
       <c r="W7" s="20"/>
       <c r="X7" s="20"/>
       <c r="Y7" s="26"/>
       <c r="Z7" s="20"/>
-      <c r="AA7" s="47"/>
-      <c r="AB7" s="37"/>
-      <c r="AC7" s="48"/>
+      <c r="AA7" s="40"/>
+      <c r="AC7" s="41"/>
     </row>
     <row r="8" ht="12.75" customHeight="1" spans="1:30">
-      <c r="A8" s="10"/>
-      <c r="B8" s="49"/>
-      <c r="C8" s="50"/>
-      <c r="D8" s="50"/>
-      <c r="E8" s="51" t="s">
+      <c r="A8" s="11"/>
+      <c r="B8" s="42"/>
+      <c r="C8" s="43"/>
+      <c r="D8" s="43"/>
+      <c r="E8" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="F8" s="52"/>
-      <c r="G8" s="53"/>
+      <c r="F8" s="45"/>
+      <c r="G8" s="46"/>
       <c r="H8" s="34"/>
       <c r="I8" s="34"/>
-      <c r="J8" s="54"/>
-      <c r="K8" s="39">
+      <c r="J8" s="47"/>
+      <c r="K8" s="37">
         <v>6245885.55000001</v>
       </c>
-      <c r="L8" s="55"/>
-      <c r="M8" s="56"/>
-      <c r="N8" s="10"/>
-      <c r="O8" s="54"/>
-      <c r="P8" s="10"/>
+      <c r="L8" s="48"/>
+      <c r="M8" s="49"/>
+      <c r="N8" s="11"/>
+      <c r="O8" s="47"/>
+      <c r="P8" s="11"/>
       <c r="Q8" s="26"/>
       <c r="R8" s="20"/>
       <c r="S8" s="20"/>
       <c r="T8" s="26"/>
       <c r="U8" s="17"/>
-      <c r="V8" s="47"/>
+      <c r="V8" s="40"/>
       <c r="W8" s="20"/>
       <c r="X8" s="20"/>
       <c r="Y8" s="26"/>
       <c r="Z8" s="20"/>
-      <c r="AA8" s="47"/>
-      <c r="AB8" s="37"/>
-      <c r="AC8" s="48"/>
+      <c r="AA8" s="40"/>
+      <c r="AC8" s="41"/>
     </row>
     <row r="9" ht="12.75" customHeight="1" spans="1:30">
-      <c r="A9" s="10"/>
-      <c r="B9" s="11"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="57"/>
+      <c r="A9" s="11"/>
+      <c r="B9" s="12"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="50"/>
       <c r="E9" s="32"/>
       <c r="F9" s="16"/>
       <c r="G9" s="18"/>
       <c r="H9" s="18"/>
       <c r="I9" s="18"/>
       <c r="J9" s="19"/>
-      <c r="K9" s="39">
+      <c r="K9" s="37">
         <v>6245885.55000001</v>
       </c>
       <c r="L9" s="21"/>
       <c r="M9" s="22"/>
       <c r="N9" s="29"/>
       <c r="O9" s="19"/>
-      <c r="P9" s="10"/>
+      <c r="P9" s="11"/>
       <c r="Q9" s="26"/>
       <c r="R9" s="20"/>
       <c r="S9" s="20"/>
       <c r="T9" s="26"/>
       <c r="U9" s="17"/>
-      <c r="V9" s="47"/>
+      <c r="V9" s="40"/>
       <c r="W9" s="20"/>
       <c r="X9" s="20"/>
       <c r="Y9" s="26"/>
       <c r="Z9" s="20"/>
-      <c r="AA9" s="47"/>
-      <c r="AB9" s="37"/>
-      <c r="AC9" s="48"/>
+      <c r="AA9" s="40"/>
+      <c r="AC9" s="41"/>
     </row>
     <row r="10" ht="12.75" customHeight="1" spans="1:30">
-      <c r="A10" s="10"/>
-      <c r="B10" s="11"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="57"/>
+      <c r="A10" s="11"/>
+      <c r="B10" s="12"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="50"/>
       <c r="E10" s="32" t="s">
         <v>31</v>
       </c>
       <c r="F10" s="16"/>
-      <c r="G10" s="58"/>
+      <c r="G10" s="51"/>
       <c r="H10" s="18"/>
       <c r="I10" s="18"/>
       <c r="J10" s="19"/>
-      <c r="K10" s="59">
-        <f t="shared" ref="K10:K17" si="0">K9+G10-J10</f>
+      <c r="K10" s="52">
+        <f t="shared" ref="K10:K20" si="0">K9+G10-J10</f>
         <v>6245885.55000001</v>
       </c>
       <c r="L10" s="21"/>
       <c r="M10" s="18"/>
       <c r="N10" s="20"/>
       <c r="O10" s="19"/>
-      <c r="P10" s="10"/>
+      <c r="P10" s="11"/>
       <c r="Q10" s="26"/>
       <c r="R10" s="20"/>
       <c r="S10" s="20"/>
       <c r="T10" s="26"/>
       <c r="U10" s="17"/>
-      <c r="V10" s="47"/>
+      <c r="V10" s="40"/>
       <c r="W10" s="20"/>
       <c r="X10" s="20"/>
       <c r="Y10" s="26"/>
       <c r="Z10" s="20"/>
-      <c r="AA10" s="47"/>
-      <c r="AB10" s="37"/>
-      <c r="AC10" s="48"/>
+      <c r="AA10" s="40"/>
+      <c r="AC10" s="41"/>
     </row>
     <row r="11" ht="12.75" customHeight="1" spans="1:30">
-      <c r="A11" s="10"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="57"/>
+      <c r="A11" s="11"/>
+      <c r="B11" s="12"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="50"/>
       <c r="E11" s="32" t="s">
         <v>32</v>
       </c>
@@ -2115,7 +2524,7 @@
       <c r="H11" s="18"/>
       <c r="I11" s="18"/>
       <c r="J11" s="19"/>
-      <c r="K11" s="59">
+      <c r="K11" s="52">
         <f t="shared" si="0"/>
         <v>6245885.55000001</v>
       </c>
@@ -2123,33 +2532,32 @@
       <c r="M11" s="18"/>
       <c r="N11" s="20"/>
       <c r="O11" s="19"/>
-      <c r="P11" s="10"/>
+      <c r="P11" s="11"/>
       <c r="Q11" s="26"/>
       <c r="R11" s="20"/>
       <c r="S11" s="20"/>
       <c r="T11" s="26"/>
       <c r="U11" s="17"/>
-      <c r="V11" s="47"/>
+      <c r="V11" s="40"/>
       <c r="W11" s="20"/>
       <c r="X11" s="20"/>
       <c r="Y11" s="26"/>
       <c r="Z11" s="20"/>
-      <c r="AA11" s="47"/>
-      <c r="AB11" s="37"/>
-      <c r="AC11" s="48"/>
+      <c r="AA11" s="40"/>
+      <c r="AC11" s="41"/>
     </row>
     <row r="12" ht="12.75" customHeight="1" spans="1:30">
-      <c r="A12" s="10"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="57"/>
+      <c r="A12" s="11"/>
+      <c r="B12" s="12"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="50"/>
       <c r="E12" s="15"/>
       <c r="F12" s="16"/>
       <c r="G12" s="18"/>
       <c r="H12" s="18"/>
       <c r="I12" s="18"/>
       <c r="J12" s="19"/>
-      <c r="K12" s="59">
+      <c r="K12" s="52">
         <f t="shared" si="0"/>
         <v>6245885.55000001</v>
       </c>
@@ -2157,28 +2565,27 @@
       <c r="M12" s="18"/>
       <c r="N12" s="20"/>
       <c r="O12" s="19"/>
-      <c r="P12" s="10"/>
+      <c r="P12" s="11"/>
       <c r="Q12" s="26"/>
       <c r="R12" s="20"/>
       <c r="S12" s="20"/>
       <c r="T12" s="26"/>
       <c r="U12" s="17"/>
-      <c r="V12" s="47"/>
+      <c r="V12" s="40"/>
       <c r="W12" s="20"/>
       <c r="X12" s="20"/>
       <c r="Y12" s="26"/>
       <c r="Z12" s="20"/>
-      <c r="AA12" s="47"/>
-      <c r="AB12" s="37"/>
-      <c r="AC12" s="48"/>
+      <c r="AA12" s="40"/>
+      <c r="AC12" s="41"/>
     </row>
     <row r="13" ht="12.75" customHeight="1" spans="1:30">
-      <c r="A13" s="10"/>
-      <c r="B13" s="60">
+      <c r="A13" s="11"/>
+      <c r="B13" s="53">
         <v>1700000</v>
       </c>
-      <c r="C13" s="10"/>
-      <c r="D13" s="57"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="50"/>
       <c r="E13" s="32" t="s">
         <v>33</v>
       </c>
@@ -2189,7 +2596,7 @@
       <c r="H13" s="18"/>
       <c r="I13" s="18"/>
       <c r="J13" s="19"/>
-      <c r="K13" s="59">
+      <c r="K13" s="52">
         <f t="shared" si="0"/>
         <v>8245885.55000001</v>
       </c>
@@ -2197,26 +2604,25 @@
       <c r="M13" s="22"/>
       <c r="N13" s="20"/>
       <c r="O13" s="19"/>
-      <c r="P13" s="10"/>
+      <c r="P13" s="11"/>
       <c r="Q13" s="26"/>
       <c r="R13" s="20"/>
       <c r="S13" s="20"/>
       <c r="T13" s="26"/>
       <c r="U13" s="17"/>
-      <c r="V13" s="47"/>
+      <c r="V13" s="40"/>
       <c r="W13" s="20"/>
       <c r="X13" s="20"/>
       <c r="Y13" s="26"/>
       <c r="Z13" s="20"/>
-      <c r="AA13" s="47"/>
-      <c r="AB13" s="37"/>
-      <c r="AC13" s="48"/>
+      <c r="AA13" s="40"/>
+      <c r="AC13" s="41"/>
     </row>
     <row r="14" ht="12.75" customHeight="1" spans="1:30">
-      <c r="A14" s="10"/>
-      <c r="B14" s="61"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="57"/>
+      <c r="A14" s="11"/>
+      <c r="B14" s="54"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="50"/>
       <c r="E14" s="32" t="s">
         <v>34</v>
       </c>
@@ -2225,7 +2631,7 @@
       <c r="H14" s="18"/>
       <c r="I14" s="18"/>
       <c r="J14" s="19"/>
-      <c r="K14" s="59">
+      <c r="K14" s="52">
         <f t="shared" si="0"/>
         <v>8245885.55000001</v>
       </c>
@@ -2233,33 +2639,32 @@
       <c r="M14" s="22"/>
       <c r="N14" s="20"/>
       <c r="O14" s="19"/>
-      <c r="P14" s="10"/>
+      <c r="P14" s="11"/>
       <c r="Q14" s="26"/>
       <c r="R14" s="20"/>
       <c r="S14" s="20"/>
       <c r="T14" s="26"/>
       <c r="U14" s="17"/>
-      <c r="V14" s="47"/>
+      <c r="V14" s="40"/>
       <c r="W14" s="20"/>
       <c r="X14" s="20"/>
       <c r="Y14" s="26"/>
       <c r="Z14" s="20"/>
-      <c r="AA14" s="47"/>
-      <c r="AB14" s="37"/>
-      <c r="AC14" s="48"/>
+      <c r="AA14" s="40"/>
+      <c r="AC14" s="41"/>
     </row>
     <row r="15" ht="12.75" customHeight="1" spans="1:30">
-      <c r="A15" s="10"/>
-      <c r="B15" s="61"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="57"/>
+      <c r="A15" s="11"/>
+      <c r="B15" s="54"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="50"/>
       <c r="E15" s="32"/>
       <c r="F15" s="16"/>
       <c r="G15" s="18"/>
       <c r="H15" s="18"/>
       <c r="I15" s="18"/>
       <c r="J15" s="19"/>
-      <c r="K15" s="59">
+      <c r="K15" s="52">
         <f t="shared" si="0"/>
         <v>8245885.55000001</v>
       </c>
@@ -2267,33 +2672,32 @@
       <c r="M15" s="22"/>
       <c r="N15" s="20"/>
       <c r="O15" s="19"/>
-      <c r="P15" s="10"/>
+      <c r="P15" s="11"/>
       <c r="Q15" s="26"/>
       <c r="R15" s="20"/>
       <c r="S15" s="20"/>
       <c r="T15" s="26"/>
       <c r="U15" s="17"/>
-      <c r="V15" s="47"/>
+      <c r="V15" s="40"/>
       <c r="W15" s="20"/>
       <c r="X15" s="20"/>
       <c r="Y15" s="26"/>
       <c r="Z15" s="20"/>
-      <c r="AA15" s="47"/>
-      <c r="AB15" s="37"/>
-      <c r="AC15" s="48"/>
+      <c r="AA15" s="40"/>
+      <c r="AC15" s="41"/>
     </row>
     <row r="16" ht="12.75" customHeight="1" spans="1:30">
-      <c r="A16" s="10"/>
-      <c r="B16" s="61"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="57"/>
+      <c r="A16" s="11"/>
+      <c r="B16" s="54"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="50"/>
       <c r="E16" s="32"/>
       <c r="F16" s="16"/>
       <c r="G16" s="18"/>
       <c r="H16" s="18"/>
       <c r="I16" s="18"/>
       <c r="J16" s="19"/>
-      <c r="K16" s="59">
+      <c r="K16" s="52">
         <f t="shared" si="0"/>
         <v>8245885.55000001</v>
       </c>
@@ -2301,66 +2705,64 @@
       <c r="M16" s="22"/>
       <c r="N16" s="20"/>
       <c r="O16" s="19"/>
-      <c r="P16" s="10"/>
+      <c r="P16" s="11"/>
       <c r="Q16" s="26"/>
       <c r="R16" s="20"/>
       <c r="S16" s="20"/>
       <c r="T16" s="26"/>
       <c r="U16" s="17"/>
-      <c r="V16" s="47"/>
+      <c r="V16" s="40"/>
       <c r="W16" s="20"/>
       <c r="X16" s="20"/>
       <c r="Y16" s="26"/>
       <c r="Z16" s="20"/>
-      <c r="AA16" s="47"/>
-      <c r="AB16" s="37"/>
-      <c r="AC16" s="48"/>
+      <c r="AA16" s="40"/>
+      <c r="AC16" s="41"/>
     </row>
-    <row r="17" ht="12.6" customHeight="1" spans="1:29">
-      <c r="A17" s="10"/>
-      <c r="B17" s="11"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="62"/>
-      <c r="E17" s="63" t="s">
+    <row r="17" ht="12.6" customHeight="1" spans="1:30">
+      <c r="A17" s="11"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="55"/>
+      <c r="E17" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="F17" s="64" t="s">
+      <c r="F17" s="57" t="s">
         <v>36</v>
       </c>
-      <c r="G17" s="65"/>
-      <c r="H17" s="65"/>
-      <c r="I17" s="65"/>
-      <c r="J17" s="66"/>
-      <c r="K17" s="59">
+      <c r="G17" s="58"/>
+      <c r="H17" s="58"/>
+      <c r="I17" s="58"/>
+      <c r="J17" s="59"/>
+      <c r="K17" s="52">
         <f t="shared" si="0"/>
         <v>8245885.55000001</v>
       </c>
-      <c r="L17" s="67"/>
+      <c r="L17" s="60"/>
       <c r="M17" s="20"/>
-      <c r="N17" s="10"/>
-      <c r="O17" s="46"/>
-      <c r="P17" s="10"/>
+      <c r="N17" s="11"/>
+      <c r="O17" s="39"/>
+      <c r="P17" s="11"/>
       <c r="Q17" s="26"/>
       <c r="R17" s="20"/>
       <c r="S17" s="20"/>
       <c r="T17" s="26"/>
       <c r="U17" s="17"/>
-      <c r="V17" s="47"/>
+      <c r="V17" s="40"/>
       <c r="W17" s="20"/>
       <c r="X17" s="20"/>
       <c r="Y17" s="26"/>
       <c r="Z17" s="20"/>
-      <c r="AA17" s="47"/>
-      <c r="AB17" s="37"/>
-      <c r="AC17" s="48"/>
+      <c r="AA17" s="40"/>
+      <c r="AC17" s="41"/>
     </row>
-    <row r="18" ht="12.6" customHeight="1" spans="1:29">
-      <c r="A18" s="10"/>
-      <c r="B18" s="11" t="s">
+    <row r="18" ht="12.6" customHeight="1" spans="1:30">
+      <c r="A18" s="11"/>
+      <c r="B18" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="C18" s="10"/>
-      <c r="D18" s="62" t="s">
+      <c r="C18" s="11"/>
+      <c r="D18" s="55" t="s">
         <v>38</v>
       </c>
       <c r="E18" s="32" t="s">
@@ -2368,70 +2770,1441 @@
       </c>
       <c r="F18" s="16"/>
       <c r="G18" s="30"/>
-      <c r="H18" s="65">
+      <c r="H18" s="58">
         <v>100000</v>
       </c>
-      <c r="I18" s="65"/>
-      <c r="J18" s="65">
+      <c r="I18" s="58"/>
+      <c r="J18" s="58">
         <v>100000</v>
       </c>
-      <c r="K18" s="59"/>
-      <c r="L18" s="68"/>
-      <c r="M18" s="57"/>
-      <c r="N18" s="10"/>
-      <c r="O18" s="69"/>
-      <c r="P18" s="10"/>
-      <c r="Q18" s="70" t="s">
+      <c r="K18" s="52">
+        <f t="shared" si="0"/>
+        <v>8145885.55000001</v>
+      </c>
+      <c r="L18" s="61"/>
+      <c r="M18" s="50"/>
+      <c r="N18" s="11"/>
+      <c r="O18" s="62"/>
+      <c r="P18" s="11"/>
+      <c r="Q18" s="63" t="s">
         <v>40</v>
       </c>
-      <c r="R18" s="70">
+      <c r="R18" s="63">
         <v>5422402</v>
       </c>
-      <c r="S18" s="70">
+      <c r="S18" s="63">
         <v>60</v>
       </c>
-      <c r="T18" s="71">
+      <c r="T18" s="64">
         <v>1933.29</v>
       </c>
-      <c r="U18" s="11" t="s">
+      <c r="U18" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="V18" s="72">
+      <c r="V18" s="65">
         <v>13081</v>
       </c>
-      <c r="W18" s="70" t="s">
+      <c r="W18" s="63" t="s">
         <v>42</v>
       </c>
-      <c r="X18" s="70" t="s">
+      <c r="X18" s="63" t="s">
         <v>43</v>
       </c>
-      <c r="Y18" s="70">
+      <c r="Y18" s="63">
         <v>4336279</v>
       </c>
-      <c r="Z18" s="70" t="s">
+      <c r="Z18" s="63" t="s">
         <v>37</v>
       </c>
-      <c r="AA18" s="70"/>
-      <c r="AB18" s="73"/>
-      <c r="AC18" s="48" t="s">
+      <c r="AA18" s="63"/>
+      <c r="AB18" s="7"/>
+      <c r="AC18" s="41" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="19" customHeight="1" spans="1:29">
-      <c r="B19" s="2" t="s">
+    <row r="19" spans="1:30">
+      <c r="B19" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="D19" s="62" t="s">
+      <c r="D19" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="E19" s="66" t="s">
+        <v>47</v>
+      </c>
+      <c r="F19" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="F19" s="3" t="s">
+      <c r="H19" s="67">
+        <v>8606.65</v>
+      </c>
+      <c r="J19" s="67">
+        <v>8606.65</v>
+      </c>
+      <c r="K19" s="52">
+        <f t="shared" si="0"/>
+        <v>8137278.90000001</v>
+      </c>
+      <c r="W19" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC19" s="10" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="20" spans="1:30">
+      <c r="B20" s="4" t="s">
         <v>45</v>
+      </c>
+      <c r="D20" s="55" t="s">
+        <v>50</v>
+      </c>
+      <c r="E20" s="66" t="s">
+        <v>51</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="H20" s="67">
+        <v>5799.85</v>
+      </c>
+      <c r="J20" s="67">
+        <v>5799.85</v>
+      </c>
+      <c r="K20" s="52">
+        <f t="shared" si="0"/>
+        <v>8131479.05000001</v>
+      </c>
+      <c r="W20" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AC20" s="10" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="21" spans="1:30">
+      <c r="A21" s="11"/>
+      <c r="B21" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D21" s="55" t="s">
+        <v>55</v>
+      </c>
+      <c r="E21" s="32" t="s">
+        <v>39</v>
+      </c>
+      <c r="F21" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="G21" s="30"/>
+      <c r="H21" s="58">
+        <v>100000</v>
+      </c>
+      <c r="I21" s="58">
+        <v>0</v>
+      </c>
+      <c r="J21" s="58">
+        <v>100000</v>
+      </c>
+      <c r="K21" s="52">
+        <f>N(K20)+N(G21)-N(J21)</f>
+        <v>8031479.05000001</v>
+      </c>
+      <c r="L21" s="61"/>
+      <c r="M21" s="50"/>
+      <c r="N21" s="11"/>
+      <c r="O21" s="62"/>
+      <c r="P21" s="11"/>
+      <c r="Q21" s="63" t="s">
+        <v>40</v>
+      </c>
+      <c r="R21" s="63" t="s">
+        <v>56</v>
+      </c>
+      <c r="S21" s="63" t="s">
+        <v>57</v>
+      </c>
+      <c r="T21" s="64">
+        <v>1933.29</v>
+      </c>
+      <c r="U21" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="V21" s="65" t="s">
+        <v>59</v>
+      </c>
+      <c r="W21" s="63" t="s">
+        <v>42</v>
+      </c>
+      <c r="X21" s="63" t="s">
+        <v>43</v>
+      </c>
+      <c r="Y21" s="63" t="s">
+        <v>60</v>
+      </c>
+      <c r="Z21" s="63" t="s">
+        <v>61</v>
+      </c>
+      <c r="AA21" s="63" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB21" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC21" s="41" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="22" spans="1:30">
+      <c r="A22" s="11"/>
+      <c r="B22" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D22" s="55" t="s">
+        <v>63</v>
+      </c>
+      <c r="E22" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="F22" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="G22" s="30"/>
+      <c r="H22" s="58">
+        <v>100000</v>
+      </c>
+      <c r="I22" s="58">
+        <v>0</v>
+      </c>
+      <c r="J22" s="58">
+        <v>100000</v>
+      </c>
+      <c r="K22" s="52">
+        <f>N(K21)+N(G22)-N(J22)</f>
+        <v>7931479.05000001</v>
+      </c>
+      <c r="L22" s="61"/>
+      <c r="M22" s="50"/>
+      <c r="N22" s="11"/>
+      <c r="O22" s="62"/>
+      <c r="P22" s="11"/>
+      <c r="Q22" s="63" t="s">
+        <v>65</v>
+      </c>
+      <c r="R22" s="63" t="s">
+        <v>66</v>
+      </c>
+      <c r="S22" s="63" t="s">
+        <v>57</v>
+      </c>
+      <c r="T22" s="64">
+        <v>1933.29</v>
+      </c>
+      <c r="U22" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="V22" s="65" t="s">
+        <v>59</v>
+      </c>
+      <c r="W22" s="63" t="s">
+        <v>52</v>
+      </c>
+      <c r="X22" s="63" t="s">
+        <v>68</v>
+      </c>
+      <c r="Y22" s="63" t="s">
+        <v>69</v>
+      </c>
+      <c r="Z22" s="63" t="s">
+        <v>70</v>
+      </c>
+      <c r="AA22" s="63" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB22" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC22" s="41" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="23" spans="1:30">
+      <c r="A23" s="11"/>
+      <c r="B23" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D23" s="55" t="s">
+        <v>72</v>
+      </c>
+      <c r="E23" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="F23" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="G23" s="30"/>
+      <c r="H23" s="58">
+        <v>95000</v>
+      </c>
+      <c r="I23" s="58">
+        <v>0</v>
+      </c>
+      <c r="J23" s="58">
+        <v>95000</v>
+      </c>
+      <c r="K23" s="52">
+        <f>N(K22)+N(G23)-N(J23)</f>
+        <v>7836479.05000001</v>
+      </c>
+      <c r="L23" s="61"/>
+      <c r="M23" s="50"/>
+      <c r="N23" s="11"/>
+      <c r="O23" s="62"/>
+      <c r="P23" s="11"/>
+      <c r="Q23" s="63" t="s">
+        <v>74</v>
+      </c>
+      <c r="R23" s="63" t="s">
+        <v>75</v>
+      </c>
+      <c r="S23" s="63" t="s">
+        <v>57</v>
+      </c>
+      <c r="T23" s="64">
+        <v>1836.62</v>
+      </c>
+      <c r="U23" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="V23" s="65" t="s">
+        <v>77</v>
+      </c>
+      <c r="W23" s="63" t="s">
+        <v>78</v>
+      </c>
+      <c r="X23" s="63" t="s">
+        <v>79</v>
+      </c>
+      <c r="Y23" s="63" t="s">
+        <v>80</v>
+      </c>
+      <c r="Z23" s="63" t="s">
+        <v>70</v>
+      </c>
+      <c r="AA23" s="63" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB23" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC23" s="41" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="24" spans="1:30">
+      <c r="A24" s="11"/>
+      <c r="B24" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D24" s="55" t="s">
+        <v>83</v>
+      </c>
+      <c r="E24" s="32" t="s">
+        <v>68</v>
+      </c>
+      <c r="F24" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="G24" s="30"/>
+      <c r="H24" s="58">
+        <v>300000</v>
+      </c>
+      <c r="I24" s="58">
+        <v>148385.54</v>
+      </c>
+      <c r="J24" s="58">
+        <v>151614.46</v>
+      </c>
+      <c r="K24" s="52">
+        <f>N(K23)+N(G24)-N(J24)</f>
+        <v>7684864.59000001</v>
+      </c>
+      <c r="L24" s="61"/>
+      <c r="M24" s="50"/>
+      <c r="N24" s="11"/>
+      <c r="O24" s="62"/>
+      <c r="P24" s="11"/>
+      <c r="Q24" s="63" t="s">
+        <v>65</v>
+      </c>
+      <c r="R24" s="63" t="s">
+        <v>69</v>
+      </c>
+      <c r="S24" s="63" t="s">
+        <v>84</v>
+      </c>
+      <c r="T24" s="64">
+        <v>9126.59</v>
+      </c>
+      <c r="U24" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="V24" s="65" t="s">
+        <v>85</v>
+      </c>
+      <c r="W24" s="63" t="s">
+        <v>52</v>
+      </c>
+      <c r="X24" s="63" t="s">
+        <v>86</v>
+      </c>
+      <c r="Y24" s="63" t="s">
+        <v>87</v>
+      </c>
+      <c r="Z24" s="63" t="s">
+        <v>88</v>
+      </c>
+      <c r="AA24" s="63" t="s">
+        <v>89</v>
+      </c>
+      <c r="AB24" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AC24" s="41" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="25" spans="1:30">
+      <c r="A25" s="11"/>
+      <c r="B25" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D25" s="55" t="s">
+        <v>92</v>
+      </c>
+      <c r="E25" s="32" t="s">
+        <v>93</v>
+      </c>
+      <c r="F25" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="G25" s="30"/>
+      <c r="H25" s="58">
+        <v>100000</v>
+      </c>
+      <c r="I25" s="58">
+        <v>50905.19</v>
+      </c>
+      <c r="J25" s="58">
+        <v>49094.81</v>
+      </c>
+      <c r="K25" s="52">
+        <f>N(K24)+N(G25)-N(J25)</f>
+        <v>7635769.78000001</v>
+      </c>
+      <c r="L25" s="61"/>
+      <c r="M25" s="50"/>
+      <c r="N25" s="11"/>
+      <c r="O25" s="62"/>
+      <c r="P25" s="11"/>
+      <c r="Q25" s="63" t="s">
+        <v>94</v>
+      </c>
+      <c r="R25" s="63" t="s">
+        <v>95</v>
+      </c>
+      <c r="S25" s="63" t="s">
+        <v>96</v>
+      </c>
+      <c r="T25" s="64">
+        <v>2348.51</v>
+      </c>
+      <c r="U25" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="V25" s="65" t="s">
+        <v>97</v>
+      </c>
+      <c r="W25" s="63" t="s">
+        <v>98</v>
+      </c>
+      <c r="X25" s="63" t="s">
+        <v>99</v>
+      </c>
+      <c r="Y25" s="63" t="s">
+        <v>100</v>
+      </c>
+      <c r="Z25" s="63" t="s">
+        <v>88</v>
+      </c>
+      <c r="AA25" s="63" t="s">
+        <v>101</v>
+      </c>
+      <c r="AB25" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AC25" s="41" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="26" s="1" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
+      <c r="A26" s="68"/>
+      <c r="B26" s="69" t="s">
+        <v>62</v>
+      </c>
+      <c r="C26" s="68"/>
+      <c r="D26" s="55" t="s">
+        <v>103</v>
+      </c>
+      <c r="E26" s="70" t="s">
+        <v>104</v>
+      </c>
+      <c r="F26" s="71"/>
+      <c r="G26" s="72"/>
+      <c r="H26" s="73">
+        <v>90000</v>
+      </c>
+      <c r="I26" s="73"/>
+      <c r="J26" s="74">
+        <v>90000</v>
+      </c>
+      <c r="K26" s="52">
+        <f t="shared" ref="K26:K38" si="1">N(K25)+N(G26)-N(J26)</f>
+        <v>7545769.78000001</v>
+      </c>
+      <c r="L26" s="75"/>
+      <c r="M26" s="76"/>
+      <c r="N26" s="68"/>
+      <c r="O26" s="77"/>
+      <c r="P26" s="68"/>
+      <c r="Q26" s="78" t="s">
+        <v>74</v>
+      </c>
+      <c r="R26" s="78">
+        <v>5375191</v>
+      </c>
+      <c r="S26" s="78">
+        <v>60</v>
+      </c>
+      <c r="T26" s="79">
+        <v>1739.96</v>
+      </c>
+      <c r="U26" s="69" t="s">
+        <v>105</v>
+      </c>
+      <c r="V26" s="80">
+        <v>13074</v>
+      </c>
+      <c r="W26" s="78" t="s">
+        <v>106</v>
+      </c>
+      <c r="X26" s="78" t="s">
+        <v>79</v>
+      </c>
+      <c r="Y26" s="78">
+        <v>4160293</v>
+      </c>
+      <c r="Z26" s="81" t="s">
+        <v>62</v>
+      </c>
+      <c r="AA26" s="63"/>
+      <c r="AB26" s="82"/>
+      <c r="AC26" s="41" t="s">
+        <v>107</v>
+      </c>
+      <c r="AD26" s="83"/>
+    </row>
+    <row r="27" s="1" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
+      <c r="A27" s="68"/>
+      <c r="B27" s="69" t="s">
+        <v>62</v>
+      </c>
+      <c r="C27" s="68"/>
+      <c r="D27" s="55" t="s">
+        <v>108</v>
+      </c>
+      <c r="E27" s="70" t="s">
+        <v>109</v>
+      </c>
+      <c r="F27" s="71"/>
+      <c r="G27" s="72"/>
+      <c r="H27" s="73">
+        <v>50000</v>
+      </c>
+      <c r="I27" s="73"/>
+      <c r="J27" s="74">
+        <v>50000</v>
+      </c>
+      <c r="K27" s="52">
+        <f t="shared" si="1"/>
+        <v>7495769.78000001</v>
+      </c>
+      <c r="L27" s="75"/>
+      <c r="M27" s="76"/>
+      <c r="N27" s="68"/>
+      <c r="O27" s="77"/>
+      <c r="P27" s="68"/>
+      <c r="Q27" s="78" t="s">
+        <v>110</v>
+      </c>
+      <c r="R27" s="78">
+        <v>5407441</v>
+      </c>
+      <c r="S27" s="78">
+        <v>60</v>
+      </c>
+      <c r="T27" s="78">
+        <v>966.65</v>
+      </c>
+      <c r="U27" s="69" t="s">
+        <v>76</v>
+      </c>
+      <c r="V27" s="80">
+        <v>13075</v>
+      </c>
+      <c r="W27" s="78" t="s">
+        <v>111</v>
+      </c>
+      <c r="X27" s="78" t="s">
+        <v>112</v>
+      </c>
+      <c r="Y27" s="78">
+        <v>5410670</v>
+      </c>
+      <c r="Z27" s="81" t="s">
+        <v>62</v>
+      </c>
+      <c r="AA27" s="63"/>
+      <c r="AB27" s="82"/>
+      <c r="AC27" s="41" t="s">
+        <v>113</v>
+      </c>
+      <c r="AD27" s="83"/>
+    </row>
+    <row r="28" s="1" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
+      <c r="A28" s="68"/>
+      <c r="B28" s="69" t="s">
+        <v>62</v>
+      </c>
+      <c r="C28" s="68"/>
+      <c r="D28" s="55" t="s">
+        <v>114</v>
+      </c>
+      <c r="E28" s="70" t="s">
+        <v>115</v>
+      </c>
+      <c r="F28" s="71"/>
+      <c r="G28" s="72"/>
+      <c r="H28" s="73">
+        <v>30000</v>
+      </c>
+      <c r="I28" s="73"/>
+      <c r="J28" s="74">
+        <v>30000</v>
+      </c>
+      <c r="K28" s="52">
+        <f t="shared" si="1"/>
+        <v>7465769.78000001</v>
+      </c>
+      <c r="L28" s="75"/>
+      <c r="M28" s="76"/>
+      <c r="N28" s="68"/>
+      <c r="O28" s="77"/>
+      <c r="P28" s="68"/>
+      <c r="Q28" s="78" t="s">
+        <v>110</v>
+      </c>
+      <c r="R28" s="78">
+        <v>5407330</v>
+      </c>
+      <c r="S28" s="78">
+        <v>60</v>
+      </c>
+      <c r="T28" s="78">
+        <v>579.99</v>
+      </c>
+      <c r="U28" s="69" t="s">
+        <v>67</v>
+      </c>
+      <c r="V28" s="80">
+        <v>13076</v>
+      </c>
+      <c r="W28" s="78" t="s">
+        <v>116</v>
+      </c>
+      <c r="X28" s="78" t="s">
+        <v>112</v>
+      </c>
+      <c r="Y28" s="78">
+        <v>5410670</v>
+      </c>
+      <c r="Z28" s="81" t="s">
+        <v>62</v>
+      </c>
+      <c r="AA28" s="63"/>
+      <c r="AB28" s="82"/>
+      <c r="AC28" s="41" t="s">
+        <v>117</v>
+      </c>
+      <c r="AD28" s="83"/>
+    </row>
+    <row r="29" s="1" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
+      <c r="A29" s="68"/>
+      <c r="B29" s="69" t="s">
+        <v>37</v>
+      </c>
+      <c r="C29" s="68"/>
+      <c r="D29" s="55" t="s">
+        <v>118</v>
+      </c>
+      <c r="E29" s="70" t="s">
+        <v>119</v>
+      </c>
+      <c r="F29" s="71"/>
+      <c r="G29" s="72"/>
+      <c r="H29" s="73">
+        <v>100000</v>
+      </c>
+      <c r="I29" s="73"/>
+      <c r="J29" s="74">
+        <v>100000</v>
+      </c>
+      <c r="K29" s="52">
+        <f t="shared" si="1"/>
+        <v>7365769.78000001</v>
+      </c>
+      <c r="L29" s="75"/>
+      <c r="M29" s="76"/>
+      <c r="N29" s="68"/>
+      <c r="O29" s="77"/>
+      <c r="P29" s="68"/>
+      <c r="Q29" s="78" t="s">
+        <v>120</v>
+      </c>
+      <c r="R29" s="78">
+        <v>4278059</v>
+      </c>
+      <c r="S29" s="78">
+        <v>60</v>
+      </c>
+      <c r="T29" s="78">
+        <v>1933.29</v>
+      </c>
+      <c r="U29" s="69" t="s">
+        <v>105</v>
+      </c>
+      <c r="V29" s="80">
+        <v>13077</v>
+      </c>
+      <c r="W29" s="78" t="s">
+        <v>121</v>
+      </c>
+      <c r="X29" s="78" t="s">
+        <v>122</v>
+      </c>
+      <c r="Y29" s="78">
+        <v>4261607</v>
+      </c>
+      <c r="Z29" s="81" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA29" s="63"/>
+      <c r="AB29" s="82"/>
+      <c r="AC29" s="41" t="s">
+        <v>123</v>
+      </c>
+      <c r="AD29" s="83"/>
+    </row>
+    <row r="30" s="1" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
+      <c r="A30" s="68"/>
+      <c r="B30" s="69" t="s">
+        <v>37</v>
+      </c>
+      <c r="C30" s="68"/>
+      <c r="D30" s="55" t="s">
+        <v>124</v>
+      </c>
+      <c r="E30" s="84" t="s">
+        <v>125</v>
+      </c>
+      <c r="F30" s="71"/>
+      <c r="G30" s="72"/>
+      <c r="H30" s="73">
+        <v>100000</v>
+      </c>
+      <c r="I30" s="72"/>
+      <c r="J30" s="73">
+        <v>100000</v>
+      </c>
+      <c r="K30" s="52">
+        <f t="shared" si="1"/>
+        <v>7265769.78000001</v>
+      </c>
+      <c r="L30" s="75"/>
+      <c r="M30" s="76"/>
+      <c r="N30" s="68"/>
+      <c r="O30" s="77"/>
+      <c r="P30" s="68"/>
+      <c r="Q30" s="78">
+        <v>500</v>
+      </c>
+      <c r="R30" s="78">
+        <v>4151323</v>
+      </c>
+      <c r="S30" s="78">
+        <v>24</v>
+      </c>
+      <c r="T30" s="78">
+        <v>4432.07</v>
+      </c>
+      <c r="U30" s="69" t="s">
+        <v>126</v>
+      </c>
+      <c r="V30" s="80">
+        <v>13078</v>
+      </c>
+      <c r="W30" s="78" t="s">
+        <v>127</v>
+      </c>
+      <c r="X30" s="78" t="s">
+        <v>128</v>
+      </c>
+      <c r="Y30" s="78">
+        <v>4149546</v>
+      </c>
+      <c r="Z30" s="81" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA30" s="63"/>
+      <c r="AB30" s="82"/>
+      <c r="AC30" s="41" t="s">
+        <v>129</v>
+      </c>
+      <c r="AD30" s="83"/>
+    </row>
+    <row r="31" s="1" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
+      <c r="A31" s="68"/>
+      <c r="B31" s="69" t="s">
+        <v>45</v>
+      </c>
+      <c r="C31" s="68"/>
+      <c r="D31" s="55" t="s">
+        <v>130</v>
+      </c>
+      <c r="E31" s="84" t="s">
+        <v>131</v>
+      </c>
+      <c r="F31" s="71" t="s">
+        <v>45</v>
+      </c>
+      <c r="G31" s="72"/>
+      <c r="H31" s="73">
+        <v>966.65</v>
+      </c>
+      <c r="I31" s="73"/>
+      <c r="J31" s="73">
+        <v>966.65</v>
+      </c>
+      <c r="K31" s="52">
+        <f t="shared" si="1"/>
+        <v>7264803.13000001</v>
+      </c>
+      <c r="L31" s="75"/>
+      <c r="M31" s="76"/>
+      <c r="N31" s="68"/>
+      <c r="O31" s="77"/>
+      <c r="P31" s="68"/>
+      <c r="Q31" s="78"/>
+      <c r="R31" s="78"/>
+      <c r="S31" s="78"/>
+      <c r="T31" s="79"/>
+      <c r="U31" s="69"/>
+      <c r="V31" s="80">
+        <v>13080</v>
+      </c>
+      <c r="W31" s="78" t="s">
+        <v>132</v>
+      </c>
+      <c r="X31" s="78"/>
+      <c r="Y31" s="78"/>
+      <c r="Z31" s="81"/>
+      <c r="AA31" s="63"/>
+      <c r="AB31" s="82"/>
+      <c r="AC31" s="41" t="s">
+        <v>133</v>
+      </c>
+      <c r="AD31" s="83"/>
+    </row>
+    <row r="32" s="1" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
+      <c r="A32" s="11"/>
+      <c r="B32" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="C32" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D32" s="55" t="s">
+        <v>134</v>
+      </c>
+      <c r="E32" s="32" t="s">
+        <v>135</v>
+      </c>
+      <c r="F32" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="G32" s="30"/>
+      <c r="H32" s="58">
+        <v>100000</v>
+      </c>
+      <c r="I32" s="58">
+        <v>61933.09</v>
+      </c>
+      <c r="J32" s="58">
+        <v>38066.91</v>
+      </c>
+      <c r="K32" s="52">
+        <f t="shared" si="1"/>
+        <v>7226736.22000001</v>
+      </c>
+      <c r="L32" s="61"/>
+      <c r="M32" s="50"/>
+      <c r="N32" s="11"/>
+      <c r="O32" s="62"/>
+      <c r="P32" s="11"/>
+      <c r="Q32" s="63" t="s">
+        <v>136</v>
+      </c>
+      <c r="R32" s="63" t="s">
+        <v>137</v>
+      </c>
+      <c r="S32" s="63" t="s">
+        <v>57</v>
+      </c>
+      <c r="T32" s="64">
+        <v>1933.29</v>
+      </c>
+      <c r="U32" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="V32" s="65" t="s">
+        <v>138</v>
+      </c>
+      <c r="W32" s="63" t="s">
+        <v>139</v>
+      </c>
+      <c r="X32" s="63" t="s">
+        <v>140</v>
+      </c>
+      <c r="Y32" s="63" t="s">
+        <v>141</v>
+      </c>
+      <c r="Z32" s="63" t="s">
+        <v>88</v>
+      </c>
+      <c r="AA32" s="63" t="s">
+        <v>101</v>
+      </c>
+      <c r="AB32" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AC32" s="41" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="33" s="1" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
+      <c r="A33" s="11"/>
+      <c r="B33" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C33" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D33" s="55" t="s">
+        <v>143</v>
+      </c>
+      <c r="E33" s="32" t="s">
+        <v>144</v>
+      </c>
+      <c r="F33" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="G33" s="30"/>
+      <c r="H33" s="58">
+        <v>100000</v>
+      </c>
+      <c r="I33" s="58">
+        <v>0</v>
+      </c>
+      <c r="J33" s="58">
+        <v>100000</v>
+      </c>
+      <c r="K33" s="52">
+        <f t="shared" si="1"/>
+        <v>7126736.22000001</v>
+      </c>
+      <c r="L33" s="61"/>
+      <c r="M33" s="50"/>
+      <c r="N33" s="11"/>
+      <c r="O33" s="62"/>
+      <c r="P33" s="11"/>
+      <c r="Q33" s="63" t="s">
+        <v>145</v>
+      </c>
+      <c r="R33" s="63" t="s">
+        <v>146</v>
+      </c>
+      <c r="S33" s="63" t="s">
+        <v>84</v>
+      </c>
+      <c r="T33" s="64">
+        <v>3042.2</v>
+      </c>
+      <c r="U33" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="V33" s="65" t="s">
+        <v>147</v>
+      </c>
+      <c r="W33" s="63" t="s">
+        <v>148</v>
+      </c>
+      <c r="X33" s="63" t="s">
+        <v>149</v>
+      </c>
+      <c r="Y33" s="63" t="s">
+        <v>150</v>
+      </c>
+      <c r="Z33" s="63" t="s">
+        <v>61</v>
+      </c>
+      <c r="AA33" s="63" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB33" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC33" s="41" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="34" s="1" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
+      <c r="A34" s="11"/>
+      <c r="B34" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="C34" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D34" s="55" t="s">
+        <v>152</v>
+      </c>
+      <c r="E34" s="32" t="s">
+        <v>153</v>
+      </c>
+      <c r="F34" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="G34" s="30"/>
+      <c r="H34" s="58">
+        <v>100000</v>
+      </c>
+      <c r="I34" s="58">
+        <v>68347.21</v>
+      </c>
+      <c r="J34" s="58">
+        <v>31652.79</v>
+      </c>
+      <c r="K34" s="52">
+        <f t="shared" si="1"/>
+        <v>7095083.43000001</v>
+      </c>
+      <c r="L34" s="61"/>
+      <c r="M34" s="50"/>
+      <c r="N34" s="11"/>
+      <c r="O34" s="62"/>
+      <c r="P34" s="11"/>
+      <c r="Q34" s="63" t="s">
+        <v>154</v>
+      </c>
+      <c r="R34" s="63" t="s">
+        <v>155</v>
+      </c>
+      <c r="S34" s="63" t="s">
+        <v>57</v>
+      </c>
+      <c r="T34" s="64">
+        <v>1933.29</v>
+      </c>
+      <c r="U34" s="12" t="s">
+        <v>156</v>
+      </c>
+      <c r="V34" s="65" t="s">
+        <v>157</v>
+      </c>
+      <c r="W34" s="63" t="s">
+        <v>48</v>
+      </c>
+      <c r="X34" s="63" t="s">
+        <v>158</v>
+      </c>
+      <c r="Y34" s="63" t="s">
+        <v>159</v>
+      </c>
+      <c r="Z34" s="63" t="s">
+        <v>88</v>
+      </c>
+      <c r="AA34" s="63" t="s">
+        <v>160</v>
+      </c>
+      <c r="AB34" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AC34" s="41" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="35" s="1" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
+      <c r="A35" s="11"/>
+      <c r="B35" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="C35" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D35" s="55" t="s">
+        <v>162</v>
+      </c>
+      <c r="E35" s="32" t="s">
+        <v>163</v>
+      </c>
+      <c r="F35" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="G35" s="30"/>
+      <c r="H35" s="58">
+        <v>50000</v>
+      </c>
+      <c r="I35" s="58">
+        <v>31774.22</v>
+      </c>
+      <c r="J35" s="58">
+        <v>18225.78</v>
+      </c>
+      <c r="K35" s="52">
+        <f t="shared" si="1"/>
+        <v>7076857.65000001</v>
+      </c>
+      <c r="L35" s="61"/>
+      <c r="M35" s="50"/>
+      <c r="N35" s="11"/>
+      <c r="O35" s="62"/>
+      <c r="P35" s="11"/>
+      <c r="Q35" s="63" t="s">
+        <v>164</v>
+      </c>
+      <c r="R35" s="63" t="s">
+        <v>165</v>
+      </c>
+      <c r="S35" s="63" t="s">
+        <v>57</v>
+      </c>
+      <c r="T35" s="64">
+        <v>966.65</v>
+      </c>
+      <c r="U35" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="V35" s="65" t="s">
+        <v>166</v>
+      </c>
+      <c r="W35" s="63" t="s">
+        <v>167</v>
+      </c>
+      <c r="X35" s="63" t="s">
+        <v>168</v>
+      </c>
+      <c r="Y35" s="63" t="s">
+        <v>169</v>
+      </c>
+      <c r="Z35" s="63" t="s">
+        <v>88</v>
+      </c>
+      <c r="AA35" s="63" t="s">
+        <v>170</v>
+      </c>
+      <c r="AB35" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AC35" s="41" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="36" s="1" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
+      <c r="A36" s="11"/>
+      <c r="B36" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C36" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D36" s="55" t="s">
+        <v>172</v>
+      </c>
+      <c r="E36" s="32" t="s">
+        <v>173</v>
+      </c>
+      <c r="F36" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="G36" s="30"/>
+      <c r="H36" s="58">
+        <v>150000</v>
+      </c>
+      <c r="I36" s="58">
+        <v>0</v>
+      </c>
+      <c r="J36" s="58">
+        <v>150000</v>
+      </c>
+      <c r="K36" s="52">
+        <f t="shared" si="1"/>
+        <v>6926857.65000001</v>
+      </c>
+      <c r="L36" s="61"/>
+      <c r="M36" s="50"/>
+      <c r="N36" s="11"/>
+      <c r="O36" s="62"/>
+      <c r="P36" s="11"/>
+      <c r="Q36" s="63" t="s">
+        <v>65</v>
+      </c>
+      <c r="R36" s="63" t="s">
+        <v>174</v>
+      </c>
+      <c r="S36" s="63" t="s">
+        <v>57</v>
+      </c>
+      <c r="T36" s="64">
+        <v>2899.93</v>
+      </c>
+      <c r="U36" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="V36" s="65" t="s">
+        <v>175</v>
+      </c>
+      <c r="W36" s="63" t="s">
+        <v>52</v>
+      </c>
+      <c r="X36" s="63" t="s">
+        <v>176</v>
+      </c>
+      <c r="Y36" s="63" t="s">
+        <v>177</v>
+      </c>
+      <c r="Z36" s="63" t="s">
+        <v>70</v>
+      </c>
+      <c r="AA36" s="63" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB36" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC36" s="41" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="37" spans="1:30">
+      <c r="B37" s="85" t="s">
+        <v>45</v>
+      </c>
+      <c r="D37" s="55" t="s">
+        <v>179</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F37" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="K37" s="52">
+        <f t="shared" si="1"/>
+        <v>6926857.65000001</v>
+      </c>
+    </row>
+    <row r="38" spans="1:30">
+      <c r="B38" s="85" t="s">
+        <v>45</v>
+      </c>
+      <c r="D38" s="55" t="s">
+        <v>180</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F38" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="K38" s="52">
+        <f t="shared" si="1"/>
+        <v>6926857.65000001</v>
+      </c>
+    </row>
+    <row r="39" s="1" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
+      <c r="A39" s="68"/>
+      <c r="B39" s="69" t="s">
+        <v>181</v>
+      </c>
+      <c r="C39" s="68"/>
+      <c r="D39" s="86" t="s">
+        <v>182</v>
+      </c>
+      <c r="E39" s="84" t="s">
+        <v>183</v>
+      </c>
+      <c r="F39" s="71" t="s">
+        <v>184</v>
+      </c>
+      <c r="G39" s="72"/>
+      <c r="H39" s="73">
+        <v>7142.86</v>
+      </c>
+      <c r="I39" s="73"/>
+      <c r="J39" s="74">
+        <v>7142.86</v>
+      </c>
+      <c r="K39" s="87">
+        <f>K38+G39-J39</f>
+        <v>6919714.79000001</v>
+      </c>
+      <c r="L39" s="75"/>
+      <c r="M39" s="76"/>
+      <c r="N39" s="68"/>
+      <c r="O39" s="77"/>
+      <c r="P39" s="68"/>
+      <c r="Q39" s="78"/>
+      <c r="R39" s="78"/>
+      <c r="S39" s="78"/>
+      <c r="T39" s="79"/>
+      <c r="U39" s="69"/>
+      <c r="V39" s="80">
+        <v>13072</v>
+      </c>
+      <c r="W39" s="78" t="s">
+        <v>52</v>
+      </c>
+      <c r="X39" s="78"/>
+      <c r="Y39" s="78"/>
+      <c r="Z39" s="81"/>
+      <c r="AA39" s="63"/>
+      <c r="AB39" s="82"/>
+      <c r="AC39" s="41"/>
+      <c r="AD39" s="83"/>
+    </row>
+    <row r="40" s="2" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
+      <c r="A40" s="88"/>
+      <c r="B40" s="89" t="s">
+        <v>62</v>
+      </c>
+      <c r="C40" s="88" t="s">
+        <v>54</v>
+      </c>
+      <c r="D40" s="90" t="s">
+        <v>185</v>
+      </c>
+      <c r="E40" s="91" t="s">
+        <v>186</v>
+      </c>
+      <c r="F40" s="92" t="s">
+        <v>54</v>
+      </c>
+      <c r="G40" s="93"/>
+      <c r="H40" s="94">
+        <v>35000</v>
+      </c>
+      <c r="I40" s="94">
+        <v>0</v>
+      </c>
+      <c r="J40" s="94">
+        <v>35000</v>
+      </c>
+      <c r="K40" s="95">
+        <f>N(K39)+N(G40)-N(J40)</f>
+        <v>6884714.79000001</v>
+      </c>
+      <c r="L40" s="96"/>
+      <c r="M40" s="97"/>
+      <c r="N40" s="88"/>
+      <c r="O40" s="98"/>
+      <c r="P40" s="88"/>
+      <c r="Q40" s="99" t="s">
+        <v>65</v>
+      </c>
+      <c r="R40" s="99" t="s">
+        <v>187</v>
+      </c>
+      <c r="S40" s="99" t="s">
+        <v>57</v>
+      </c>
+      <c r="T40" s="100">
+        <v>676.65</v>
+      </c>
+      <c r="U40" s="89" t="s">
+        <v>41</v>
+      </c>
+      <c r="V40" s="101" t="s">
+        <v>188</v>
+      </c>
+      <c r="W40" s="99" t="s">
+        <v>52</v>
+      </c>
+      <c r="X40" s="99" t="s">
+        <v>189</v>
+      </c>
+      <c r="Y40" s="99" t="s">
+        <v>190</v>
+      </c>
+      <c r="Z40" s="99" t="s">
+        <v>70</v>
+      </c>
+      <c r="AA40" s="99" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB40" s="102" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC40" s="103" t="s">
+        <v>191</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A39">
+    <cfRule type="containsText" dxfId="0" priority="6" operator="between" text="OK">
+      <formula>NOT(ISERROR(SEARCH("OK",A39)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="5" operator="between" text="w/ docs">
+      <formula>NOT(ISERROR(SEARCH("w/ docs",A39)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="4" operator="between" text="w/ docs for checking">
+      <formula>NOT(ISERROR(SEARCH("w/ docs for checking",A39)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1"/>
   <headerFooter/>

</xml_diff>

<commit_message>
Redesign dashboard with responsive iOS-style layout
</commit_message>
<xml_diff>
--- a/provident-system/server/uploads/templates/sl.xlsx
+++ b/provident-system/server/uploads/templates/sl.xlsx
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="231">
   <si>
     <t>SUBSIDIARY LEDGER</t>
   </si>
@@ -636,6 +636,123 @@
   </si>
   <si>
     <t>0085135996</t>
+  </si>
+  <si>
+    <t>2026-06-4278</t>
+  </si>
+  <si>
+    <t>GUILAS, SHERYLL ANN S.</t>
+  </si>
+  <si>
+    <t>4160848</t>
+  </si>
+  <si>
+    <t>13081</t>
+  </si>
+  <si>
+    <t>GUILAS, GEORGE JOSE MARIA C.</t>
+  </si>
+  <si>
+    <t>4673905</t>
+  </si>
+  <si>
+    <t>2908217/ 2908168</t>
+  </si>
+  <si>
+    <t>MAY</t>
+  </si>
+  <si>
+    <t>0085171399</t>
+  </si>
+  <si>
+    <t>2026-06-4279</t>
+  </si>
+  <si>
+    <t>ISIP, AIDA M.</t>
+  </si>
+  <si>
+    <t>500</t>
+  </si>
+  <si>
+    <t>4151206</t>
+  </si>
+  <si>
+    <t>REGISTRAR I</t>
+  </si>
+  <si>
+    <t>13082</t>
+  </si>
+  <si>
+    <t>SAN MATIAS NHS/ STO. TOMAS</t>
+  </si>
+  <si>
+    <t>BASILIO, CARINA I.</t>
+  </si>
+  <si>
+    <t>41501964</t>
+  </si>
+  <si>
+    <t>2908163</t>
+  </si>
+  <si>
+    <t>0085069110</t>
+  </si>
+  <si>
+    <t>2026-06-4280</t>
+  </si>
+  <si>
+    <t>MARTIN, PAOLA P.</t>
+  </si>
+  <si>
+    <t>5398880</t>
+  </si>
+  <si>
+    <t>T-II</t>
+  </si>
+  <si>
+    <t>13083</t>
+  </si>
+  <si>
+    <t>MORALES, ALONA L.</t>
+  </si>
+  <si>
+    <t>4593317</t>
+  </si>
+  <si>
+    <t>2908088</t>
+  </si>
+  <si>
+    <t>1525075199</t>
+  </si>
+  <si>
+    <t>2026-06-4281</t>
+  </si>
+  <si>
+    <t>PONCE, CARINA P.</t>
+  </si>
+  <si>
+    <t>4149963</t>
+  </si>
+  <si>
+    <t>HT-I</t>
+  </si>
+  <si>
+    <t>13084</t>
+  </si>
+  <si>
+    <t>GULAP HS/ CANDABA</t>
+  </si>
+  <si>
+    <t>BACALA, EDMON G.</t>
+  </si>
+  <si>
+    <t>4263120</t>
+  </si>
+  <si>
+    <t>2907841/ 2907942</t>
+  </si>
+  <si>
+    <t>0085067818</t>
   </si>
 </sst>
 </file>
@@ -973,7 +1090,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -989,12 +1106,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1384,7 +1495,7 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1408,16 +1519,16 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="6" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="7" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="7" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="8" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="5" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="6" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="7" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -1426,85 +1537,85 @@
     <xf numFmtId="0" fontId="35" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="36" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="40" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="39" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="39" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="40" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="40" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="39" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="39" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="40" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="40" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="39" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="39" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="40" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="40" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="39" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="39" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="40" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="40" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="39" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="39" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="40" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="40" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="39" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1745,52 +1856,52 @@
     <xf numFmtId="43" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="43" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="43" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="43" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="43" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
@@ -2128,7 +2239,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:AD40"/>
+  <dimension ref="A1:AD44"/>
   <sheetFormatPr defaultColWidth="14.4444444444444" defaultRowHeight="15.6" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="8.22222222222222" style="3" customWidth="1"/>
@@ -4193,6 +4304,310 @@
         <v>191</v>
       </c>
     </row>
+    <row r="41" s="2" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
+      <c r="A41" s="11"/>
+      <c r="B41" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="C41" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D41" s="55" t="s">
+        <v>192</v>
+      </c>
+      <c r="E41" s="32" t="s">
+        <v>193</v>
+      </c>
+      <c r="F41" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="G41" s="30"/>
+      <c r="H41" s="58">
+        <v>125000</v>
+      </c>
+      <c r="I41" s="58">
+        <v>93264.14</v>
+      </c>
+      <c r="J41" s="58">
+        <v>31735.86</v>
+      </c>
+      <c r="K41" s="52">
+        <f>N(K40)+N(G41)-N(J41)</f>
+        <v>6852978.93000001</v>
+      </c>
+      <c r="L41" s="61"/>
+      <c r="M41" s="50"/>
+      <c r="N41" s="11"/>
+      <c r="O41" s="62"/>
+      <c r="P41" s="11"/>
+      <c r="Q41" s="63" t="s">
+        <v>65</v>
+      </c>
+      <c r="R41" s="63" t="s">
+        <v>194</v>
+      </c>
+      <c r="S41" s="63" t="s">
+        <v>57</v>
+      </c>
+      <c r="T41" s="64">
+        <v>2416.62</v>
+      </c>
+      <c r="U41" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="V41" s="65" t="s">
+        <v>195</v>
+      </c>
+      <c r="W41" s="63" t="s">
+        <v>52</v>
+      </c>
+      <c r="X41" s="63" t="s">
+        <v>196</v>
+      </c>
+      <c r="Y41" s="63" t="s">
+        <v>197</v>
+      </c>
+      <c r="Z41" s="63" t="s">
+        <v>88</v>
+      </c>
+      <c r="AA41" s="63" t="s">
+        <v>198</v>
+      </c>
+      <c r="AB41" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="AC41" s="41" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="42" s="2" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
+      <c r="A42" s="11"/>
+      <c r="B42" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="C42" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D42" s="55" t="s">
+        <v>201</v>
+      </c>
+      <c r="E42" s="32" t="s">
+        <v>202</v>
+      </c>
+      <c r="F42" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="G42" s="30"/>
+      <c r="H42" s="58">
+        <v>100000</v>
+      </c>
+      <c r="I42" s="58">
+        <v>69930.85</v>
+      </c>
+      <c r="J42" s="58">
+        <v>30069.15</v>
+      </c>
+      <c r="K42" s="52">
+        <f>N(K41)+N(G42)-N(J42)</f>
+        <v>6822909.78000001</v>
+      </c>
+      <c r="L42" s="61"/>
+      <c r="M42" s="50"/>
+      <c r="N42" s="11"/>
+      <c r="O42" s="62"/>
+      <c r="P42" s="11"/>
+      <c r="Q42" s="63" t="s">
+        <v>203</v>
+      </c>
+      <c r="R42" s="63" t="s">
+        <v>204</v>
+      </c>
+      <c r="S42" s="63" t="s">
+        <v>57</v>
+      </c>
+      <c r="T42" s="64">
+        <v>1933.29</v>
+      </c>
+      <c r="U42" s="12" t="s">
+        <v>205</v>
+      </c>
+      <c r="V42" s="65" t="s">
+        <v>206</v>
+      </c>
+      <c r="W42" s="63" t="s">
+        <v>207</v>
+      </c>
+      <c r="X42" s="63" t="s">
+        <v>208</v>
+      </c>
+      <c r="Y42" s="63" t="s">
+        <v>209</v>
+      </c>
+      <c r="Z42" s="63" t="s">
+        <v>88</v>
+      </c>
+      <c r="AA42" s="63" t="s">
+        <v>210</v>
+      </c>
+      <c r="AB42" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AC42" s="41" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="43" s="2" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
+      <c r="A43" s="11"/>
+      <c r="B43" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="C43" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D43" s="55" t="s">
+        <v>212</v>
+      </c>
+      <c r="E43" s="32" t="s">
+        <v>213</v>
+      </c>
+      <c r="F43" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="G43" s="30"/>
+      <c r="H43" s="58">
+        <v>100000</v>
+      </c>
+      <c r="I43" s="58">
+        <v>65156.15</v>
+      </c>
+      <c r="J43" s="58">
+        <v>34843.85</v>
+      </c>
+      <c r="K43" s="52">
+        <f>N(K42)+N(G43)-N(J43)</f>
+        <v>6788065.93000001</v>
+      </c>
+      <c r="L43" s="61"/>
+      <c r="M43" s="50"/>
+      <c r="N43" s="11"/>
+      <c r="O43" s="62"/>
+      <c r="P43" s="11"/>
+      <c r="Q43" s="63" t="s">
+        <v>164</v>
+      </c>
+      <c r="R43" s="63" t="s">
+        <v>214</v>
+      </c>
+      <c r="S43" s="63" t="s">
+        <v>57</v>
+      </c>
+      <c r="T43" s="64">
+        <v>1933.29</v>
+      </c>
+      <c r="U43" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="V43" s="65" t="s">
+        <v>216</v>
+      </c>
+      <c r="W43" s="63" t="s">
+        <v>167</v>
+      </c>
+      <c r="X43" s="63" t="s">
+        <v>217</v>
+      </c>
+      <c r="Y43" s="63" t="s">
+        <v>218</v>
+      </c>
+      <c r="Z43" s="63" t="s">
+        <v>88</v>
+      </c>
+      <c r="AA43" s="63" t="s">
+        <v>219</v>
+      </c>
+      <c r="AB43" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AC43" s="41" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="44" s="2" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
+      <c r="A44" s="11"/>
+      <c r="B44" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="C44" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D44" s="55" t="s">
+        <v>221</v>
+      </c>
+      <c r="E44" s="32" t="s">
+        <v>222</v>
+      </c>
+      <c r="F44" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="G44" s="30"/>
+      <c r="H44" s="58">
+        <v>100000</v>
+      </c>
+      <c r="I44" s="58">
+        <v>44059.91</v>
+      </c>
+      <c r="J44" s="58">
+        <v>55940.09</v>
+      </c>
+      <c r="K44" s="52">
+        <f>N(K43)+N(G44)-N(J44)</f>
+        <v>6732125.84000001</v>
+      </c>
+      <c r="L44" s="61"/>
+      <c r="M44" s="50"/>
+      <c r="N44" s="11"/>
+      <c r="O44" s="62"/>
+      <c r="P44" s="11"/>
+      <c r="Q44" s="63" t="s">
+        <v>154</v>
+      </c>
+      <c r="R44" s="63" t="s">
+        <v>223</v>
+      </c>
+      <c r="S44" s="63" t="s">
+        <v>57</v>
+      </c>
+      <c r="T44" s="64">
+        <v>1933.29</v>
+      </c>
+      <c r="U44" s="12" t="s">
+        <v>224</v>
+      </c>
+      <c r="V44" s="65" t="s">
+        <v>225</v>
+      </c>
+      <c r="W44" s="63" t="s">
+        <v>226</v>
+      </c>
+      <c r="X44" s="63" t="s">
+        <v>227</v>
+      </c>
+      <c r="Y44" s="63" t="s">
+        <v>228</v>
+      </c>
+      <c r="Z44" s="63" t="s">
+        <v>88</v>
+      </c>
+      <c r="AA44" s="63" t="s">
+        <v>229</v>
+      </c>
+      <c r="AB44" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AC44" s="41" t="s">
+        <v>230</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="A39">
     <cfRule type="containsText" dxfId="0" priority="6" operator="between" text="OK">

</xml_diff>

<commit_message>
Complete dashboard redesign and template management workflow
</commit_message>
<xml_diff>
--- a/provident-system/server/uploads/templates/sl.xlsx
+++ b/provident-system/server/uploads/templates/sl.xlsx
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="302">
   <si>
     <t>SUBSIDIARY LEDGER</t>
   </si>
@@ -602,9 +602,27 @@
     <t>2026-06-4274</t>
   </si>
   <si>
+    <t>MARCELO, JANET B.</t>
+  </si>
+  <si>
+    <t>Refund</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>0085103288</t>
+  </si>
+  <si>
     <t>2026-06-4275</t>
   </si>
   <si>
+    <t>GUILAS, SHERYLL ANN S.</t>
+  </si>
+  <si>
+    <t>0085171399</t>
+  </si>
+  <si>
     <t>SALARY</t>
   </si>
   <si>
@@ -629,9 +647,6 @@
     <t>13080</t>
   </si>
   <si>
-    <t>N/A</t>
-  </si>
-  <si>
     <t>0</t>
   </si>
   <si>
@@ -641,9 +656,6 @@
     <t>2026-06-4278</t>
   </si>
   <si>
-    <t>GUILAS, SHERYLL ANN S.</t>
-  </si>
-  <si>
     <t>4160848</t>
   </si>
   <si>
@@ -662,9 +674,6 @@
     <t>MAY</t>
   </si>
   <si>
-    <t>0085171399</t>
-  </si>
-  <si>
     <t>2026-06-4279</t>
   </si>
   <si>
@@ -753,6 +762,210 @@
   </si>
   <si>
     <t>0085067818</t>
+  </si>
+  <si>
+    <t>2026-06-4282</t>
+  </si>
+  <si>
+    <t>CARLOS, MA. CORAZON Q.</t>
+  </si>
+  <si>
+    <t>002</t>
+  </si>
+  <si>
+    <t>5383356</t>
+  </si>
+  <si>
+    <t>13086</t>
+  </si>
+  <si>
+    <t>JOSE ESCALER MS/ APALIT</t>
+  </si>
+  <si>
+    <t>BALAGTAS, JOYCE A.</t>
+  </si>
+  <si>
+    <t>4160504</t>
+  </si>
+  <si>
+    <t>2908091</t>
+  </si>
+  <si>
+    <t>3425042474</t>
+  </si>
+  <si>
+    <t>2026-06-4283</t>
+  </si>
+  <si>
+    <t>NOLASCO, SHEREE ANN P.</t>
+  </si>
+  <si>
+    <t>5394419</t>
+  </si>
+  <si>
+    <t>13087</t>
+  </si>
+  <si>
+    <t>SABANILLA ES/ MEXICO SOUTH</t>
+  </si>
+  <si>
+    <t>CHAN, MARY GRACE B.</t>
+  </si>
+  <si>
+    <t>4674039</t>
+  </si>
+  <si>
+    <t>0085196022</t>
+  </si>
+  <si>
+    <t>2026-06-4284</t>
+  </si>
+  <si>
+    <t>FLORES, JONNEL M.</t>
+  </si>
+  <si>
+    <t>578</t>
+  </si>
+  <si>
+    <t>4263240</t>
+  </si>
+  <si>
+    <t>HT-III</t>
+  </si>
+  <si>
+    <t>13088</t>
+  </si>
+  <si>
+    <t>DIOSDADO MACAPAGAL HS/ MEXICO</t>
+  </si>
+  <si>
+    <t>LOZANO, AL M.</t>
+  </si>
+  <si>
+    <t>5376565</t>
+  </si>
+  <si>
+    <t>2908143</t>
+  </si>
+  <si>
+    <t>0085072340</t>
+  </si>
+  <si>
+    <t>2026-06-4285</t>
+  </si>
+  <si>
+    <t>QUIZON, ROSE ANNE N.</t>
+  </si>
+  <si>
+    <t>580</t>
+  </si>
+  <si>
+    <t>5399328</t>
+  </si>
+  <si>
+    <t>13089</t>
+  </si>
+  <si>
+    <t>TINAJERO NHS/ ANNEX MAGALANG</t>
+  </si>
+  <si>
+    <t>ALA, DAISY B.</t>
+  </si>
+  <si>
+    <t>5380970</t>
+  </si>
+  <si>
+    <t>2908044</t>
+  </si>
+  <si>
+    <t>1975049244</t>
+  </si>
+  <si>
+    <t>2026-06-4288</t>
+  </si>
+  <si>
+    <t>SARIFA, DARLENE G.</t>
+  </si>
+  <si>
+    <t>4160464</t>
+  </si>
+  <si>
+    <t>13090</t>
+  </si>
+  <si>
+    <t>SAN ESTEBAN ES/ MACABEBE</t>
+  </si>
+  <si>
+    <t>ISIP, ALVIN D.</t>
+  </si>
+  <si>
+    <t>4261047</t>
+  </si>
+  <si>
+    <t>3425033823</t>
+  </si>
+  <si>
+    <t>2026-06-4289</t>
+  </si>
+  <si>
+    <t>VERAN, JHON LEVIN S.</t>
+  </si>
+  <si>
+    <t>5435671</t>
+  </si>
+  <si>
+    <t>13091</t>
+  </si>
+  <si>
+    <t>PAGUINTO, CARLITO C.</t>
+  </si>
+  <si>
+    <t>4162628</t>
+  </si>
+  <si>
+    <t>4605012448</t>
+  </si>
+  <si>
+    <t>2026-06-4290</t>
+  </si>
+  <si>
+    <t>FLORES, JOANNA Y.</t>
+  </si>
+  <si>
+    <t>4667054</t>
+  </si>
+  <si>
+    <t>T-I</t>
+  </si>
+  <si>
+    <t>13092</t>
+  </si>
+  <si>
+    <t>MACARAYO, MICHELLE T.</t>
+  </si>
+  <si>
+    <t>4277016</t>
+  </si>
+  <si>
+    <t>2908111</t>
+  </si>
+  <si>
+    <t>0085161687</t>
+  </si>
+  <si>
+    <t>2026-06-4291</t>
+  </si>
+  <si>
+    <t>13085</t>
+  </si>
+  <si>
+    <t>CANLAS, EMILIANA D.</t>
+  </si>
+  <si>
+    <t>4260758</t>
+  </si>
+  <si>
+    <t>0085176897</t>
   </si>
 </sst>
 </file>
@@ -1296,7 +1509,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -1358,19 +1571,6 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="hair">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="hair">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="hair">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -1495,7 +1695,7 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1507,34 +1707,34 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="5" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="6" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="6" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="7" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="7" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1619,7 +1819,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1847,15 +2047,9 @@
     <xf numFmtId="0" fontId="20" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="43" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -1876,9 +2070,6 @@
     </xf>
     <xf numFmtId="43" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="43" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -2239,7 +2430,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:AD44"/>
+  <dimension ref="A1:AD52"/>
   <sheetFormatPr defaultColWidth="14.4444444444444" defaultRowHeight="15.6" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="8.22222222222222" style="3" customWidth="1"/>
@@ -4141,56 +4332,172 @@
         <v>178</v>
       </c>
     </row>
-    <row r="37" spans="1:30">
-      <c r="B37" s="85" t="s">
+    <row r="37" s="2" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
+      <c r="A37" s="11"/>
+      <c r="B37" s="12" t="s">
         <v>45</v>
+      </c>
+      <c r="C37" s="11" t="s">
+        <v>54</v>
       </c>
       <c r="D37" s="55" t="s">
         <v>179</v>
       </c>
-      <c r="E37" s="3" t="s">
+      <c r="E37" s="32" t="s">
+        <v>180</v>
+      </c>
+      <c r="F37" s="16" t="s">
+        <v>181</v>
+      </c>
+      <c r="G37" s="30"/>
+      <c r="H37" s="58">
+        <v>6908.77</v>
+      </c>
+      <c r="I37" s="58">
+        <v>0</v>
+      </c>
+      <c r="J37" s="58">
+        <v>6908.77</v>
+      </c>
+      <c r="K37" s="52">
+        <f t="shared" ref="K37:K52" si="2">N(K36)+N(G37)-N(J37)</f>
+        <v>6919948.88000001</v>
+      </c>
+      <c r="L37" s="61"/>
+      <c r="M37" s="50"/>
+      <c r="N37" s="11"/>
+      <c r="O37" s="62"/>
+      <c r="P37" s="11"/>
+      <c r="Q37" s="63" t="s">
+        <v>182</v>
+      </c>
+      <c r="R37" s="63" t="s">
+        <v>182</v>
+      </c>
+      <c r="S37" s="63" t="s">
+        <v>182</v>
+      </c>
+      <c r="T37" s="64">
+        <v>0</v>
+      </c>
+      <c r="U37" s="12" t="s">
+        <v>182</v>
+      </c>
+      <c r="V37" s="65" t="s">
+        <v>182</v>
+      </c>
+      <c r="W37" s="63" t="s">
+        <v>52</v>
+      </c>
+      <c r="X37" s="63" t="s">
+        <v>182</v>
+      </c>
+      <c r="Y37" s="63" t="s">
+        <v>182</v>
+      </c>
+      <c r="Z37" s="63" t="s">
+        <v>181</v>
+      </c>
+      <c r="AA37" s="63" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB37" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC37" s="41" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="38" s="2" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
+      <c r="A38" s="11"/>
+      <c r="B38" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="F37" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="K37" s="52">
-        <f t="shared" si="1"/>
-        <v>6926857.65000001</v>
-      </c>
-    </row>
-    <row r="38" spans="1:30">
-      <c r="B38" s="85" t="s">
-        <v>45</v>
+      <c r="C38" s="11" t="s">
+        <v>54</v>
       </c>
       <c r="D38" s="55" t="s">
-        <v>180</v>
-      </c>
-      <c r="E38" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="F38" s="5" t="s">
-        <v>45</v>
+        <v>184</v>
+      </c>
+      <c r="E38" s="32" t="s">
+        <v>185</v>
+      </c>
+      <c r="F38" s="16" t="s">
+        <v>181</v>
+      </c>
+      <c r="G38" s="30"/>
+      <c r="H38" s="58">
+        <v>4349.91</v>
+      </c>
+      <c r="I38" s="58">
+        <v>0</v>
+      </c>
+      <c r="J38" s="58">
+        <v>4349.91</v>
       </c>
       <c r="K38" s="52">
-        <f t="shared" si="1"/>
-        <v>6926857.65000001</v>
+        <f t="shared" si="2"/>
+        <v>6915598.97000001</v>
+      </c>
+      <c r="L38" s="61"/>
+      <c r="M38" s="50"/>
+      <c r="N38" s="11"/>
+      <c r="O38" s="62"/>
+      <c r="P38" s="11"/>
+      <c r="Q38" s="63" t="s">
+        <v>182</v>
+      </c>
+      <c r="R38" s="63" t="s">
+        <v>182</v>
+      </c>
+      <c r="S38" s="63" t="s">
+        <v>182</v>
+      </c>
+      <c r="T38" s="64">
+        <v>0</v>
+      </c>
+      <c r="U38" s="12" t="s">
+        <v>182</v>
+      </c>
+      <c r="V38" s="65" t="s">
+        <v>182</v>
+      </c>
+      <c r="W38" s="63" t="s">
+        <v>52</v>
+      </c>
+      <c r="X38" s="63" t="s">
+        <v>182</v>
+      </c>
+      <c r="Y38" s="63" t="s">
+        <v>182</v>
+      </c>
+      <c r="Z38" s="63" t="s">
+        <v>181</v>
+      </c>
+      <c r="AA38" s="63" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB38" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC38" s="41" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="39" s="1" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
       <c r="A39" s="68"/>
       <c r="B39" s="69" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="C39" s="68"/>
-      <c r="D39" s="86" t="s">
-        <v>182</v>
+      <c r="D39" s="85" t="s">
+        <v>188</v>
       </c>
       <c r="E39" s="84" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="F39" s="71" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="G39" s="72"/>
       <c r="H39" s="73">
@@ -4200,9 +4507,9 @@
       <c r="J39" s="74">
         <v>7142.86</v>
       </c>
-      <c r="K39" s="87">
-        <f>K38+G39-J39</f>
-        <v>6919714.79000001</v>
+      <c r="K39" s="52">
+        <f t="shared" si="2"/>
+        <v>6908456.11000001</v>
       </c>
       <c r="L39" s="75"/>
       <c r="M39" s="76"/>
@@ -4229,79 +4536,79 @@
       <c r="AD39" s="83"/>
     </row>
     <row r="40" s="2" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
-      <c r="A40" s="88"/>
-      <c r="B40" s="89" t="s">
+      <c r="A40" s="86"/>
+      <c r="B40" s="87" t="s">
         <v>62</v>
       </c>
-      <c r="C40" s="88" t="s">
-        <v>54</v>
-      </c>
-      <c r="D40" s="90" t="s">
-        <v>185</v>
-      </c>
-      <c r="E40" s="91" t="s">
-        <v>186</v>
-      </c>
-      <c r="F40" s="92" t="s">
-        <v>54</v>
-      </c>
-      <c r="G40" s="93"/>
-      <c r="H40" s="94">
+      <c r="C40" s="86" t="s">
+        <v>54</v>
+      </c>
+      <c r="D40" s="88" t="s">
+        <v>191</v>
+      </c>
+      <c r="E40" s="89" t="s">
+        <v>192</v>
+      </c>
+      <c r="F40" s="90" t="s">
+        <v>54</v>
+      </c>
+      <c r="G40" s="91"/>
+      <c r="H40" s="92">
         <v>35000</v>
       </c>
-      <c r="I40" s="94">
+      <c r="I40" s="92">
         <v>0</v>
       </c>
-      <c r="J40" s="94">
+      <c r="J40" s="92">
         <v>35000</v>
       </c>
-      <c r="K40" s="95">
-        <f>N(K39)+N(G40)-N(J40)</f>
-        <v>6884714.79000001</v>
-      </c>
-      <c r="L40" s="96"/>
-      <c r="M40" s="97"/>
-      <c r="N40" s="88"/>
-      <c r="O40" s="98"/>
-      <c r="P40" s="88"/>
-      <c r="Q40" s="99" t="s">
+      <c r="K40" s="52">
+        <f t="shared" si="2"/>
+        <v>6873456.11000001</v>
+      </c>
+      <c r="L40" s="93"/>
+      <c r="M40" s="94"/>
+      <c r="N40" s="86"/>
+      <c r="O40" s="95"/>
+      <c r="P40" s="86"/>
+      <c r="Q40" s="96" t="s">
         <v>65</v>
       </c>
-      <c r="R40" s="99" t="s">
-        <v>187</v>
-      </c>
-      <c r="S40" s="99" t="s">
+      <c r="R40" s="96" t="s">
+        <v>193</v>
+      </c>
+      <c r="S40" s="96" t="s">
         <v>57</v>
       </c>
-      <c r="T40" s="100">
+      <c r="T40" s="97">
         <v>676.65</v>
       </c>
-      <c r="U40" s="89" t="s">
+      <c r="U40" s="87" t="s">
         <v>41</v>
       </c>
-      <c r="V40" s="101" t="s">
-        <v>188</v>
-      </c>
-      <c r="W40" s="99" t="s">
+      <c r="V40" s="98" t="s">
+        <v>194</v>
+      </c>
+      <c r="W40" s="96" t="s">
         <v>52</v>
       </c>
-      <c r="X40" s="99" t="s">
-        <v>189</v>
-      </c>
-      <c r="Y40" s="99" t="s">
-        <v>190</v>
-      </c>
-      <c r="Z40" s="99" t="s">
+      <c r="X40" s="96" t="s">
+        <v>182</v>
+      </c>
+      <c r="Y40" s="96" t="s">
+        <v>195</v>
+      </c>
+      <c r="Z40" s="96" t="s">
         <v>70</v>
       </c>
-      <c r="AA40" s="99" t="s">
-        <v>54</v>
-      </c>
-      <c r="AB40" s="102" t="s">
-        <v>54</v>
-      </c>
-      <c r="AC40" s="103" t="s">
-        <v>191</v>
+      <c r="AA40" s="96" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB40" s="99" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC40" s="100" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="41" s="2" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
@@ -4313,10 +4620,10 @@
         <v>54</v>
       </c>
       <c r="D41" s="55" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="E41" s="32" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="F41" s="16" t="s">
         <v>54</v>
@@ -4332,8 +4639,8 @@
         <v>31735.86</v>
       </c>
       <c r="K41" s="52">
-        <f>N(K40)+N(G41)-N(J41)</f>
-        <v>6852978.93000001</v>
+        <f t="shared" si="2"/>
+        <v>6841720.25000001</v>
       </c>
       <c r="L41" s="61"/>
       <c r="M41" s="50"/>
@@ -4344,7 +4651,7 @@
         <v>65</v>
       </c>
       <c r="R41" s="63" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="S41" s="63" t="s">
         <v>57</v>
@@ -4356,28 +4663,28 @@
         <v>41</v>
       </c>
       <c r="V41" s="65" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="W41" s="63" t="s">
         <v>52</v>
       </c>
       <c r="X41" s="63" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="Y41" s="63" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="Z41" s="63" t="s">
         <v>88</v>
       </c>
       <c r="AA41" s="63" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="AB41" s="7" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="AC41" s="41" t="s">
-        <v>200</v>
+        <v>186</v>
       </c>
     </row>
     <row r="42" s="2" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
@@ -4389,10 +4696,10 @@
         <v>54</v>
       </c>
       <c r="D42" s="55" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="E42" s="32" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="F42" s="16" t="s">
         <v>54</v>
@@ -4408,8 +4715,8 @@
         <v>30069.15</v>
       </c>
       <c r="K42" s="52">
-        <f>N(K41)+N(G42)-N(J42)</f>
-        <v>6822909.78000001</v>
+        <f t="shared" si="2"/>
+        <v>6811651.10000001</v>
       </c>
       <c r="L42" s="61"/>
       <c r="M42" s="50"/>
@@ -4417,10 +4724,10 @@
       <c r="O42" s="62"/>
       <c r="P42" s="11"/>
       <c r="Q42" s="63" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="R42" s="63" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="S42" s="63" t="s">
         <v>57</v>
@@ -4429,31 +4736,31 @@
         <v>1933.29</v>
       </c>
       <c r="U42" s="12" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="V42" s="65" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="W42" s="63" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="X42" s="63" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="Y42" s="63" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="Z42" s="63" t="s">
         <v>88</v>
       </c>
       <c r="AA42" s="63" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="AB42" s="7" t="s">
         <v>90</v>
       </c>
       <c r="AC42" s="41" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
     </row>
     <row r="43" s="2" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
@@ -4465,10 +4772,10 @@
         <v>54</v>
       </c>
       <c r="D43" s="55" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="E43" s="32" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="F43" s="16" t="s">
         <v>54</v>
@@ -4484,8 +4791,8 @@
         <v>34843.85</v>
       </c>
       <c r="K43" s="52">
-        <f>N(K42)+N(G43)-N(J43)</f>
-        <v>6788065.93000001</v>
+        <f t="shared" si="2"/>
+        <v>6776807.25000001</v>
       </c>
       <c r="L43" s="61"/>
       <c r="M43" s="50"/>
@@ -4496,7 +4803,7 @@
         <v>164</v>
       </c>
       <c r="R43" s="63" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="S43" s="63" t="s">
         <v>57</v>
@@ -4505,31 +4812,31 @@
         <v>1933.29</v>
       </c>
       <c r="U43" s="12" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="V43" s="65" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="W43" s="63" t="s">
         <v>167</v>
       </c>
       <c r="X43" s="63" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="Y43" s="63" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="Z43" s="63" t="s">
         <v>88</v>
       </c>
       <c r="AA43" s="63" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="AB43" s="7" t="s">
         <v>90</v>
       </c>
       <c r="AC43" s="41" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="44" s="2" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
@@ -4541,10 +4848,10 @@
         <v>54</v>
       </c>
       <c r="D44" s="55" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="E44" s="32" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="F44" s="16" t="s">
         <v>54</v>
@@ -4560,8 +4867,8 @@
         <v>55940.09</v>
       </c>
       <c r="K44" s="52">
-        <f>N(K43)+N(G44)-N(J44)</f>
-        <v>6732125.84000001</v>
+        <f t="shared" si="2"/>
+        <v>6720867.16000001</v>
       </c>
       <c r="L44" s="61"/>
       <c r="M44" s="50"/>
@@ -4572,7 +4879,7 @@
         <v>154</v>
       </c>
       <c r="R44" s="63" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="S44" s="63" t="s">
         <v>57</v>
@@ -4581,31 +4888,639 @@
         <v>1933.29</v>
       </c>
       <c r="U44" s="12" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="V44" s="65" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="W44" s="63" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="X44" s="63" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="Y44" s="63" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="Z44" s="63" t="s">
         <v>88</v>
       </c>
       <c r="AA44" s="63" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="AB44" s="7" t="s">
         <v>90</v>
       </c>
       <c r="AC44" s="41" t="s">
-        <v>230</v>
+        <v>233</v>
+      </c>
+    </row>
+    <row r="45" s="2" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
+      <c r="A45" s="11"/>
+      <c r="B45" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="C45" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D45" s="55" t="s">
+        <v>234</v>
+      </c>
+      <c r="E45" s="32" t="s">
+        <v>235</v>
+      </c>
+      <c r="F45" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="G45" s="30"/>
+      <c r="H45" s="58">
+        <v>100000</v>
+      </c>
+      <c r="I45" s="58">
+        <v>65156.15</v>
+      </c>
+      <c r="J45" s="58">
+        <v>34843.85</v>
+      </c>
+      <c r="K45" s="52">
+        <f t="shared" si="2"/>
+        <v>6686023.31000001</v>
+      </c>
+      <c r="L45" s="61"/>
+      <c r="M45" s="50"/>
+      <c r="N45" s="11"/>
+      <c r="O45" s="62"/>
+      <c r="P45" s="11"/>
+      <c r="Q45" s="63" t="s">
+        <v>236</v>
+      </c>
+      <c r="R45" s="63" t="s">
+        <v>237</v>
+      </c>
+      <c r="S45" s="63" t="s">
+        <v>57</v>
+      </c>
+      <c r="T45" s="64">
+        <v>1933.29</v>
+      </c>
+      <c r="U45" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="V45" s="65" t="s">
+        <v>238</v>
+      </c>
+      <c r="W45" s="63" t="s">
+        <v>239</v>
+      </c>
+      <c r="X45" s="63" t="s">
+        <v>240</v>
+      </c>
+      <c r="Y45" s="63" t="s">
+        <v>241</v>
+      </c>
+      <c r="Z45" s="63" t="s">
+        <v>88</v>
+      </c>
+      <c r="AA45" s="63" t="s">
+        <v>242</v>
+      </c>
+      <c r="AB45" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AC45" s="41" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="46" s="2" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
+      <c r="A46" s="11"/>
+      <c r="B46" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C46" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D46" s="55" t="s">
+        <v>244</v>
+      </c>
+      <c r="E46" s="32" t="s">
+        <v>245</v>
+      </c>
+      <c r="F46" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="G46" s="30"/>
+      <c r="H46" s="58">
+        <v>100000</v>
+      </c>
+      <c r="I46" s="58">
+        <v>0</v>
+      </c>
+      <c r="J46" s="58">
+        <v>100000</v>
+      </c>
+      <c r="K46" s="52">
+        <f t="shared" si="2"/>
+        <v>6586023.31000001</v>
+      </c>
+      <c r="L46" s="61"/>
+      <c r="M46" s="50"/>
+      <c r="N46" s="11"/>
+      <c r="O46" s="62"/>
+      <c r="P46" s="11"/>
+      <c r="Q46" s="63" t="s">
+        <v>120</v>
+      </c>
+      <c r="R46" s="63" t="s">
+        <v>246</v>
+      </c>
+      <c r="S46" s="63" t="s">
+        <v>84</v>
+      </c>
+      <c r="T46" s="64">
+        <v>3042.2</v>
+      </c>
+      <c r="U46" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="V46" s="65" t="s">
+        <v>247</v>
+      </c>
+      <c r="W46" s="63" t="s">
+        <v>248</v>
+      </c>
+      <c r="X46" s="63" t="s">
+        <v>249</v>
+      </c>
+      <c r="Y46" s="63" t="s">
+        <v>250</v>
+      </c>
+      <c r="Z46" s="63" t="s">
+        <v>70</v>
+      </c>
+      <c r="AA46" s="63" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB46" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC46" s="41" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="47" s="2" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
+      <c r="A47" s="11"/>
+      <c r="B47" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="C47" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D47" s="55" t="s">
+        <v>252</v>
+      </c>
+      <c r="E47" s="32" t="s">
+        <v>253</v>
+      </c>
+      <c r="F47" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="G47" s="30"/>
+      <c r="H47" s="58">
+        <v>100000</v>
+      </c>
+      <c r="I47" s="58">
+        <v>69930.85</v>
+      </c>
+      <c r="J47" s="58">
+        <v>30069.15</v>
+      </c>
+      <c r="K47" s="52">
+        <f t="shared" si="2"/>
+        <v>6555954.16000001</v>
+      </c>
+      <c r="L47" s="61"/>
+      <c r="M47" s="50"/>
+      <c r="N47" s="11"/>
+      <c r="O47" s="62"/>
+      <c r="P47" s="11"/>
+      <c r="Q47" s="63" t="s">
+        <v>254</v>
+      </c>
+      <c r="R47" s="63" t="s">
+        <v>255</v>
+      </c>
+      <c r="S47" s="63" t="s">
+        <v>96</v>
+      </c>
+      <c r="T47" s="64">
+        <v>2348.51</v>
+      </c>
+      <c r="U47" s="12" t="s">
+        <v>256</v>
+      </c>
+      <c r="V47" s="65" t="s">
+        <v>257</v>
+      </c>
+      <c r="W47" s="63" t="s">
+        <v>258</v>
+      </c>
+      <c r="X47" s="63" t="s">
+        <v>259</v>
+      </c>
+      <c r="Y47" s="63" t="s">
+        <v>260</v>
+      </c>
+      <c r="Z47" s="63" t="s">
+        <v>88</v>
+      </c>
+      <c r="AA47" s="63" t="s">
+        <v>261</v>
+      </c>
+      <c r="AB47" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AC47" s="41" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="48" s="2" customFormat="1" ht="12.6" customHeight="1" spans="1:30">
+      <c r="A48" s="11"/>
+      <c r="B48" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="C48" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D48" s="55" t="s">
+        <v>263</v>
+      </c>
+      <c r="E48" s="32" t="s">
+        <v>264</v>
+      </c>
+      <c r="F48" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="G48" s="30"/>
+      <c r="H48" s="58">
+        <v>100000</v>
+      </c>
+      <c r="I48" s="58">
+        <v>58677.73</v>
+      </c>
+      <c r="J48" s="58">
+        <v>41322.27</v>
+      </c>
+      <c r="K48" s="52">
+        <f t="shared" si="2"/>
+        <v>6514631.89000001</v>
+      </c>
+      <c r="L48" s="61"/>
+      <c r="M48" s="50"/>
+      <c r="N48" s="11"/>
+      <c r="O48" s="62"/>
+      <c r="P48" s="11"/>
+      <c r="Q48" s="63" t="s">
+        <v>265</v>
+      </c>
+      <c r="R48" s="63" t="s">
+        <v>266</v>
+      </c>
+      <c r="S48" s="63" t="s">
+        <v>57</v>
+      </c>
+      <c r="T48" s="64">
+        <v>1933.29</v>
+      </c>
+      <c r="U48" s="12" t="s">
+        <v>156</v>
+      </c>
+      <c r="V48" s="65" t="s">
+        <v>267</v>
+      </c>
+      <c r="W48" s="63" t="s">
+        <v>268</v>
+      </c>
+      <c r="X48" s="63" t="s">
+        <v>269</v>
+      </c>
+      <c r="Y48" s="63" t="s">
+        <v>270</v>
+      </c>
+      <c r="Z48" s="63" t="s">
+        <v>88</v>
+      </c>
+      <c r="AA48" s="63" t="s">
+        <v>271</v>
+      </c>
+      <c r="AB48" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AC48" s="41" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="49" s="2" customFormat="1" ht="12.6" customHeight="1" spans="1:29">
+      <c r="A49" s="11"/>
+      <c r="B49" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C49" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D49" s="55" t="s">
+        <v>273</v>
+      </c>
+      <c r="E49" s="32" t="s">
+        <v>274</v>
+      </c>
+      <c r="F49" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="G49" s="30"/>
+      <c r="H49" s="58">
+        <v>100000</v>
+      </c>
+      <c r="I49" s="58">
+        <v>0</v>
+      </c>
+      <c r="J49" s="58">
+        <v>100000</v>
+      </c>
+      <c r="K49" s="52">
+        <f t="shared" si="2"/>
+        <v>6414631.89000001</v>
+      </c>
+      <c r="L49" s="61"/>
+      <c r="M49" s="50"/>
+      <c r="N49" s="11"/>
+      <c r="O49" s="62"/>
+      <c r="P49" s="11"/>
+      <c r="Q49" s="63" t="s">
+        <v>110</v>
+      </c>
+      <c r="R49" s="63" t="s">
+        <v>275</v>
+      </c>
+      <c r="S49" s="63" t="s">
+        <v>57</v>
+      </c>
+      <c r="T49" s="64">
+        <v>1933.29</v>
+      </c>
+      <c r="U49" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="V49" s="65" t="s">
+        <v>276</v>
+      </c>
+      <c r="W49" s="63" t="s">
+        <v>277</v>
+      </c>
+      <c r="X49" s="63" t="s">
+        <v>278</v>
+      </c>
+      <c r="Y49" s="63" t="s">
+        <v>279</v>
+      </c>
+      <c r="Z49" s="63" t="s">
+        <v>61</v>
+      </c>
+      <c r="AA49" s="63" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB49" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC49" s="41" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="50" s="2" customFormat="1" ht="12.6" customHeight="1" spans="1:29">
+      <c r="A50" s="11"/>
+      <c r="B50" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C50" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D50" s="55" t="s">
+        <v>281</v>
+      </c>
+      <c r="E50" s="32" t="s">
+        <v>282</v>
+      </c>
+      <c r="F50" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="G50" s="30"/>
+      <c r="H50" s="58">
+        <v>100000</v>
+      </c>
+      <c r="I50" s="58">
+        <v>0</v>
+      </c>
+      <c r="J50" s="58">
+        <v>100000</v>
+      </c>
+      <c r="K50" s="52">
+        <f t="shared" si="2"/>
+        <v>6314631.89000001</v>
+      </c>
+      <c r="L50" s="61"/>
+      <c r="M50" s="50"/>
+      <c r="N50" s="11"/>
+      <c r="O50" s="62"/>
+      <c r="P50" s="11"/>
+      <c r="Q50" s="63" t="s">
+        <v>154</v>
+      </c>
+      <c r="R50" s="63" t="s">
+        <v>283</v>
+      </c>
+      <c r="S50" s="63" t="s">
+        <v>57</v>
+      </c>
+      <c r="T50" s="64">
+        <v>1933.29</v>
+      </c>
+      <c r="U50" s="12" t="s">
+        <v>156</v>
+      </c>
+      <c r="V50" s="65" t="s">
+        <v>284</v>
+      </c>
+      <c r="W50" s="63" t="s">
+        <v>48</v>
+      </c>
+      <c r="X50" s="63" t="s">
+        <v>285</v>
+      </c>
+      <c r="Y50" s="63" t="s">
+        <v>286</v>
+      </c>
+      <c r="Z50" s="63" t="s">
+        <v>61</v>
+      </c>
+      <c r="AA50" s="63" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB50" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC50" s="41" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="51" s="2" customFormat="1" ht="12.6" customHeight="1" spans="1:29">
+      <c r="A51" s="11"/>
+      <c r="B51" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="C51" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D51" s="55" t="s">
+        <v>288</v>
+      </c>
+      <c r="E51" s="32" t="s">
+        <v>289</v>
+      </c>
+      <c r="F51" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="G51" s="30"/>
+      <c r="H51" s="58">
+        <v>100000</v>
+      </c>
+      <c r="I51" s="58">
+        <v>66755.66</v>
+      </c>
+      <c r="J51" s="58">
+        <v>33244.34</v>
+      </c>
+      <c r="K51" s="52">
+        <f t="shared" si="2"/>
+        <v>6281387.55000001</v>
+      </c>
+      <c r="L51" s="61"/>
+      <c r="M51" s="50"/>
+      <c r="N51" s="11"/>
+      <c r="O51" s="62"/>
+      <c r="P51" s="11"/>
+      <c r="Q51" s="63" t="s">
+        <v>154</v>
+      </c>
+      <c r="R51" s="63" t="s">
+        <v>290</v>
+      </c>
+      <c r="S51" s="63" t="s">
+        <v>57</v>
+      </c>
+      <c r="T51" s="64">
+        <v>1933.29</v>
+      </c>
+      <c r="U51" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="V51" s="65" t="s">
+        <v>292</v>
+      </c>
+      <c r="W51" s="63" t="s">
+        <v>48</v>
+      </c>
+      <c r="X51" s="63" t="s">
+        <v>293</v>
+      </c>
+      <c r="Y51" s="63" t="s">
+        <v>294</v>
+      </c>
+      <c r="Z51" s="63" t="s">
+        <v>88</v>
+      </c>
+      <c r="AA51" s="63" t="s">
+        <v>295</v>
+      </c>
+      <c r="AB51" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AC51" s="41" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="52" s="2" customFormat="1" ht="12.6" customHeight="1" spans="1:29">
+      <c r="A52" s="11"/>
+      <c r="B52" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="C52" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D52" s="55" t="s">
+        <v>297</v>
+      </c>
+      <c r="E52" s="32" t="s">
+        <v>168</v>
+      </c>
+      <c r="F52" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="G52" s="30"/>
+      <c r="H52" s="58">
+        <v>100000</v>
+      </c>
+      <c r="I52" s="58">
+        <v>67527.44</v>
+      </c>
+      <c r="J52" s="58">
+        <v>32472.56</v>
+      </c>
+      <c r="K52" s="52">
+        <f t="shared" si="2"/>
+        <v>6248914.99000001</v>
+      </c>
+      <c r="L52" s="61"/>
+      <c r="M52" s="50"/>
+      <c r="N52" s="11"/>
+      <c r="O52" s="62"/>
+      <c r="P52" s="11"/>
+      <c r="Q52" s="63" t="s">
+        <v>164</v>
+      </c>
+      <c r="R52" s="63" t="s">
+        <v>169</v>
+      </c>
+      <c r="S52" s="63" t="s">
+        <v>57</v>
+      </c>
+      <c r="T52" s="64">
+        <v>1933.29</v>
+      </c>
+      <c r="U52" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="V52" s="65" t="s">
+        <v>298</v>
+      </c>
+      <c r="W52" s="63" t="s">
+        <v>167</v>
+      </c>
+      <c r="X52" s="63" t="s">
+        <v>299</v>
+      </c>
+      <c r="Y52" s="63" t="s">
+        <v>300</v>
+      </c>
+      <c r="Z52" s="63" t="s">
+        <v>88</v>
+      </c>
+      <c r="AA52" s="63" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB52" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC52" s="41" t="s">
+        <v>301</v>
       </c>
     </row>
   </sheetData>

</xml_diff>